<commit_message>
Enriquece leads com dominios e checagem Data Stone
</commit_message>
<xml_diff>
--- a/formacao/atividades-feitas/levantamento-influenciadores-e-leads-automotivos-patagon-ai-2026-10.xlsx
+++ b/formacao/atividades-feitas/levantamento-influenciadores-e-leads-automotivos-patagon-ai-2026-10.xlsx
@@ -2,11 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R6fdfce1c9937476d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Influenciadores e fontes" sheetId="2" r:id="R6b0aff5b10484006"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads candidatos" sheetId="3" r:id="Rf294de30737d4fe8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revisão manual" sheetId="4" r:id="Rdaade7b982f94476"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pesquisa pública 15" sheetId="5" r:id="R029c33ead9ef4741"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Rba54ecee92674e59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Influenciadores e fontes" sheetId="2" r:id="R3c75c32480224378"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads candidatos" sheetId="3" r:id="R4687d97842dd4b37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revisão manual" sheetId="4" r:id="R350b2b1154764c40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pesquisa pública 15" sheetId="5" r:id="Ree5bb8a1d9e54aae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enriquecimento público" sheetId="20" r:id="R31c10ed8a8824e2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Stone - domínios" sheetId="21" r:id="R49ff7b94a18f4278"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Stone - pessoas" sheetId="22" r:id="R94b7e849c8c3469f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,6 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="2">
+    <x:numFmt numFmtId="200" formatCode="@"/>
+    <x:numFmt numFmtId="201" formatCode="00000000000000"/>
+  </x:numFmts>
   <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
@@ -63,12 +70,92 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="20">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17233D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE85B10"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17233D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE85B10"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17233D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE85B10"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17233D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE85B10"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17233D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE85B10"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17233D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE85B10"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17233D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE85B10"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17233D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE85B10"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -180,7 +267,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="56">
+  <x:cellXfs count="227">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -305,6 +392,397 @@
     <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -402,6 +880,61 @@
     <x:tableColumn id="7" name="Fontes públicas"/>
     <x:tableColumn id="8" name="Leitura ICP / pendência"/>
     <x:tableColumn id="9" name="Data Stone"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="EnriquecimentoPublicoPatagon" displayName="EnriquecimentoPublicoPatagon" ref="A5:M57" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:M57"/>
+  <x:tableColumns count="13">
+    <x:tableColumn id="1" name="Nome"/>
+    <x:tableColumn id="2" name="Instagram"/>
+    <x:tableColumn id="3" name="Empresa informada no lead"/>
+    <x:tableColumn id="4" name="Domínio/site da empresa"/>
+    <x:tableColumn id="5" name="Cargo/vínculo da pessoa"/>
+    <x:tableColumn id="6" name="E-mail profissional individual"/>
+    <x:tableColumn id="7" name="Celular/WhatsApp profissional público"/>
+    <x:tableColumn id="8" name="Canal geral da empresa (não pessoal)"/>
+    <x:tableColumn id="9" name="Fonte do domínio/empresa"/>
+    <x:tableColumn id="10" name="Fonte pública do perfil"/>
+    <x:tableColumn id="11" name="Status de verificação"/>
+    <x:tableColumn id="12" name="Resultado da busca da pessoa"/>
+    <x:tableColumn id="13" name="Notas e limites"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="DataStoneDominiosPatagon" displayName="DataStoneDominiosPatagon" ref="A5:H30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:H30"/>
+  <x:tableColumns count="8">
+    <x:tableColumn id="1" name="Domínio consultado na Data Stone"/>
+    <x:tableColumn id="2" name="Empresa(s) associadas aos leads"/>
+    <x:tableColumn id="3" name="Resultados da API"/>
+    <x:tableColumn id="4" name="CNPJ candidato(s) por nome"/>
+    <x:tableColumn id="5" name="Razão social / nome fantasia correspondente"/>
+    <x:tableColumn id="6" name="Cidade(s) / UF"/>
+    <x:tableColumn id="7" name="Status da correspondência"/>
+    <x:tableColumn id="8" name="Observação"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="DataStonePessoasPatagon" displayName="DataStonePessoasPatagon" ref="A5:G57" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:G57"/>
+  <x:tableColumns count="7">
+    <x:tableColumn id="1" name="Lead"/>
+    <x:tableColumn id="2" name="Instagram"/>
+    <x:tableColumn id="3" name="Empresa/domain candidato"/>
+    <x:tableColumn id="4" name="Resultado da busca nominal Data Stone"/>
+    <x:tableColumn id="5" name="E-mail individual retornado pela API"/>
+    <x:tableColumn id="6" name="Celular individual retornado pela API"/>
+    <x:tableColumn id="7" name="Interpretação / próximo passo"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -8886,7 +9419,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d51409de2ac46f4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1aa411758bb45bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11880,7 +12413,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3550c0fab5094208"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb76a138fafb4deb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12299,7 +12832,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5a5da3c801e439f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re720891ccf5c490d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12843,7 +13376,3610 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fe5f42467284a43"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6467faff8f8740bf"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="56" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="34" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="31" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="58" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="58" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="44" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="42" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="62" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="92" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="209" t="str">
+        <x:v>Enriquecimento público · domínio e contato</x:v>
+      </x:c>
+      <x:c r="B1" s="209"/>
+      <x:c r="C1" s="209"/>
+      <x:c r="D1" s="209"/>
+      <x:c r="E1" s="209"/>
+      <x:c r="F1" s="209"/>
+      <x:c r="G1" s="209"/>
+      <x:c r="H1" s="209"/>
+      <x:c r="I1" s="209"/>
+      <x:c r="J1" s="209"/>
+      <x:c r="K1" s="209"/>
+      <x:c r="L1" s="209"/>
+      <x:c r="M1" s="209"/>
+    </x:row>
+    <x:row r="2" ht="34" customHeight="1">
+      <x:c r="A2" s="6" t="str">
+        <x:v>Pesquisa de 52 leads automotivos. Domínio ≠ vínculo confirmado; contatos corporativos ficam separados de e-mail/celular individual. Nenhum e-mail foi inferido. Atualizado em 08/10/2026.</x:v>
+      </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+      <x:c r="H2" s="6"/>
+      <x:c r="I2" s="6"/>
+      <x:c r="J2" s="6"/>
+      <x:c r="K2" s="6"/>
+      <x:c r="L2" s="6"/>
+      <x:c r="M2" s="6"/>
+    </x:row>
+    <x:row r="5" ht="42" customHeight="1">
+      <x:c r="A5" s="221" t="str">
+        <x:v>Nome</x:v>
+      </x:c>
+      <x:c r="B5" s="222" t="str">
+        <x:v>Instagram</x:v>
+      </x:c>
+      <x:c r="C5" s="222" t="str">
+        <x:v>Empresa informada no lead</x:v>
+      </x:c>
+      <x:c r="D5" s="222" t="str">
+        <x:v>Domínio/site da empresa</x:v>
+      </x:c>
+      <x:c r="E5" s="222" t="str">
+        <x:v>Cargo/vínculo da pessoa</x:v>
+      </x:c>
+      <x:c r="F5" s="222" t="str">
+        <x:v>E-mail profissional individual</x:v>
+      </x:c>
+      <x:c r="G5" s="222" t="str">
+        <x:v>Celular/WhatsApp profissional público</x:v>
+      </x:c>
+      <x:c r="H5" s="222" t="str">
+        <x:v>Canal geral da empresa (não pessoal)</x:v>
+      </x:c>
+      <x:c r="I5" s="222" t="str">
+        <x:v>Fonte do domínio/empresa</x:v>
+      </x:c>
+      <x:c r="J5" s="222" t="str">
+        <x:v>Fonte pública do perfil</x:v>
+      </x:c>
+      <x:c r="K5" s="222" t="str">
+        <x:v>Status de verificação</x:v>
+      </x:c>
+      <x:c r="L5" s="222" t="str">
+        <x:v>Resultado da busca da pessoa</x:v>
+      </x:c>
+      <x:c r="M5" s="223" t="str">
+        <x:v>Notas e limites</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="56" customHeight="1">
+      <x:c r="A6" s="51" t="str">
+        <x:v>Thiago Pinho</x:v>
+      </x:c>
+      <x:c r="B6" s="51" t="str">
+        <x:v>@thiagopinhotiti</x:v>
+      </x:c>
+      <x:c r="C6" s="51" t="str">
+        <x:v>Pinho Concessionária de Seminovos / Grupo S Pinho</x:v>
+      </x:c>
+      <x:c r="D6" s="51" t="str">
+        <x:v>pinhoveiculos.com (link da bio; associação nominal pendente)</x:v>
+      </x:c>
+      <x:c r="E6" s="51" t="str">
+        <x:v>Empresário / presidente</x:v>
+      </x:c>
+      <x:c r="F6" s="51" t="str"/>
+      <x:c r="G6" s="51" t="str"/>
+      <x:c r="H6" s="51" t="str">
+        <x:v>(51) 3731-3912; contato@pinhoveiculos.com — site Pinho Veículos (Rio Pardo), associação com o lead não confirmada</x:v>
+      </x:c>
+      <x:c r="I6" s="51" t="str">
+        <x:v>https://pinhoveiculos.com/empresa.html</x:v>
+      </x:c>
+      <x:c r="J6" s="51" t="str">
+        <x:v>https://www.instagram.com/thiagopinhotiti</x:v>
+      </x:c>
+      <x:c r="K6" s="51" t="str">
+        <x:v>Domínio identificado; vínculo/unidade individual parcial ou pendente</x:v>
+      </x:c>
+      <x:c r="L6" s="51" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M6" s="51" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. O lead indica Pinho Seminovos/Grupo S Pinho e aponta para pinhoveiculos.com. Há um site de concessionária Chevrolet Pinho homônima, mas não há evidência suficiente para vincular este lead à rede autorizada.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="56" customHeight="1">
+      <x:c r="A7" s="52" t="str">
+        <x:v>Eltton Andradee</x:v>
+      </x:c>
+      <x:c r="B7" s="52" t="str">
+        <x:v>@elttonandradee</x:v>
+      </x:c>
+      <x:c r="C7" s="52" t="str">
+        <x:v>TAG Veículos</x:v>
+      </x:c>
+      <x:c r="D7" s="52" t="str">
+        <x:v>tagveiculosdf.com.br</x:v>
+      </x:c>
+      <x:c r="E7" s="52" t="str">
+        <x:v>Empresário</x:v>
+      </x:c>
+      <x:c r="F7" s="52" t="str"/>
+      <x:c r="G7" s="52" t="str">
+        <x:v>5561991510770</x:v>
+      </x:c>
+      <x:c r="H7" s="52" t="str">
+        <x:v>(61) 99253-1206; tagveiculosdf@gmail.com — site oficial</x:v>
+      </x:c>
+      <x:c r="I7" s="52" t="str">
+        <x:v>https://tagveiculosdf.com.br/</x:v>
+      </x:c>
+      <x:c r="J7" s="52" t="str">
+        <x:v>https://www.instagram.com/elttonandradee</x:v>
+      </x:c>
+      <x:c r="K7" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L7" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M7" s="52" t="str">
+        <x:v>Número/WhatsApp divulgado na bio/link público do próprio perfil; não validado pela empresa.. Site oficial identifica Tag Veículos em Brasília; oferta de novos e seminovos, não comprova concessionária autorizada de marca.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="56" customHeight="1">
+      <x:c r="A8" s="52" t="str">
+        <x:v>SANDRA CARVALHO ⛤</x:v>
+      </x:c>
+      <x:c r="B8" s="52" t="str">
+        <x:v>@sandra.carvalho0702</x:v>
+      </x:c>
+      <x:c r="C8" s="52" t="str">
+        <x:v>AK Auto Center</x:v>
+      </x:c>
+      <x:c r="D8" s="52" t="str">
+        <x:v>akautocenter.com.br</x:v>
+      </x:c>
+      <x:c r="E8" s="52" t="str">
+        <x:v>Diretora Executiva</x:v>
+      </x:c>
+      <x:c r="F8" s="52" t="str"/>
+      <x:c r="G8" s="52" t="str"/>
+      <x:c r="H8" s="52" t="str">
+        <x:v>(11) 5184-0935 / (11) 5041-0429; atendimento@akautocenter.com.br — site oficial</x:v>
+      </x:c>
+      <x:c r="I8" s="52" t="str">
+        <x:v>https://www.akautocenter.com.br/contato/</x:v>
+      </x:c>
+      <x:c r="J8" s="52" t="str">
+        <x:v>https://www.instagram.com/sandra.carvalho0702</x:v>
+      </x:c>
+      <x:c r="K8" s="52" t="str">
+        <x:v>Domínio confirmado; vínculo da pessoa apoiado por fonte pública nominal</x:v>
+      </x:c>
+      <x:c r="L8" s="52" t="str">
+        <x:v>Perfil declara Diretora Executiva da AK Auto Center; evidência profissional independente também a identifica como sócia/proprietária.</x:v>
+      </x:c>
+      <x:c r="M8" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Site oficial e contato da AK Auto Center em São Paulo; fonte pública externa identifica Sandra Carvalho como sócia-proprietária. É oficina multimarcas, não concessionária OEM.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="56" customHeight="1">
+      <x:c r="A9" s="52" t="str">
+        <x:v>Jaime Campelo Bessa</x:v>
+      </x:c>
+      <x:c r="B9" s="52" t="str">
+        <x:v>@jaimedapro</x:v>
+      </x:c>
+      <x:c r="C9" s="52" t="str">
+        <x:v>Pro Veículos Manaus / Alugue na Pro / Alveam</x:v>
+      </x:c>
+      <x:c r="D9" s="52" t="str">
+        <x:v>proveiculosmanaus.com.br</x:v>
+      </x:c>
+      <x:c r="E9" s="52" t="str">
+        <x:v>Profissional / empresário automotivo</x:v>
+      </x:c>
+      <x:c r="F9" s="52" t="str"/>
+      <x:c r="G9" s="52" t="str"/>
+      <x:c r="H9" s="52" t="str">
+        <x:v>(92) 98147-7000; (92) 99320-5084 — site oficial</x:v>
+      </x:c>
+      <x:c r="I9" s="52" t="str">
+        <x:v>https://www.proveiculosmanaus.com.br/</x:v>
+      </x:c>
+      <x:c r="J9" s="52" t="str">
+        <x:v>https://www.instagram.com/jaimedapro</x:v>
+      </x:c>
+      <x:c r="K9" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L9" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M9" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Site oficial em Manaus; estoque contém veículos de várias marcas, portanto não atende ao critério de concessionária monomarca autorizada. Empresa encontrada, vínculo nominal do lead não confirmado.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="56" customHeight="1">
+      <x:c r="A10" s="52" t="str">
+        <x:v>Dallyane Barbosa Costa</x:v>
+      </x:c>
+      <x:c r="B10" s="52" t="str">
+        <x:v>@dallyanecostahonda</x:v>
+      </x:c>
+      <x:c r="C10" s="52" t="str">
+        <x:v>Alagoas Motos</x:v>
+      </x:c>
+      <x:c r="D10" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="E10" s="52" t="str">
+        <x:v>Coordenadora Web / F&amp;I</x:v>
+      </x:c>
+      <x:c r="F10" s="52" t="str"/>
+      <x:c r="G10" s="52" t="str">
+        <x:v>558299960571</x:v>
+      </x:c>
+      <x:c r="H10" s="52" t="str">
+        <x:v>(82) 3539-8605; WhatsApp geral (82) 99996-0571 — site oficial</x:v>
+      </x:c>
+      <x:c r="I10" s="52" t="str">
+        <x:v>https://alagoasmotos.com.br/</x:v>
+      </x:c>
+      <x:c r="J10" s="52" t="str">
+        <x:v>https://www.instagram.com/dallyanecostahonda</x:v>
+      </x:c>
+      <x:c r="K10" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L10" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M10" s="52" t="str">
+        <x:v>Número/WhatsApp divulgado na bio/link público do próprio perfil; não validado pela empresa.. Site oficial Honda; lista Arapiraca, Maceió e União dos Palmares (3 lojas em AL). LinkedIn corporativo informa vínculo com Pernambuco Motos e outras unidades do grupo, mas validar se a prospecção será pela empresa local ou grupo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="56" customHeight="1">
+      <x:c r="A11" s="52" t="str">
+        <x:v>Deyvid Bezerra</x:v>
+      </x:c>
+      <x:c r="B11" s="52" t="str">
+        <x:v>@deyvid.honda</x:v>
+      </x:c>
+      <x:c r="C11" s="52" t="str">
+        <x:v>Alagoas Motos</x:v>
+      </x:c>
+      <x:c r="D11" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="E11" s="52" t="str">
+        <x:v>Coordenador de Vendas</x:v>
+      </x:c>
+      <x:c r="F11" s="52" t="str"/>
+      <x:c r="G11" s="52" t="str">
+        <x:v>5582998184800</x:v>
+      </x:c>
+      <x:c r="H11" s="52" t="str">
+        <x:v>(82) 3539-8605; WhatsApp geral (82) 99996-0571 — site oficial</x:v>
+      </x:c>
+      <x:c r="I11" s="52" t="str">
+        <x:v>https://alagoasmotos.com.br/</x:v>
+      </x:c>
+      <x:c r="J11" s="52" t="str">
+        <x:v>https://www.instagram.com/deyvid.honda</x:v>
+      </x:c>
+      <x:c r="K11" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L11" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M11" s="52" t="str">
+        <x:v>Número/WhatsApp divulgado na bio/link público do próprio perfil; não validado pela empresa.. Site oficial Honda; lista Arapiraca, Maceió e União dos Palmares (3 lojas em AL). LinkedIn corporativo informa vínculo com Pernambuco Motos e outras unidades do grupo, mas validar se a prospecção será pela empresa local ou grupo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="56" customHeight="1">
+      <x:c r="A12" s="52" t="str">
+        <x:v>Emerson Angelino Cavalcante</x:v>
+      </x:c>
+      <x:c r="B12" s="52" t="str">
+        <x:v>@emerson.honda</x:v>
+      </x:c>
+      <x:c r="C12" s="52" t="str">
+        <x:v>Alagoas Motos</x:v>
+      </x:c>
+      <x:c r="D12" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="E12" s="52" t="str">
+        <x:v>Gerente de Consórcio e instrutor</x:v>
+      </x:c>
+      <x:c r="F12" s="52" t="str"/>
+      <x:c r="G12" s="52" t="str">
+        <x:v>5582999890705</x:v>
+      </x:c>
+      <x:c r="H12" s="52" t="str">
+        <x:v>(82) 3539-8605; WhatsApp geral (82) 99996-0571 — site oficial</x:v>
+      </x:c>
+      <x:c r="I12" s="52" t="str">
+        <x:v>https://alagoasmotos.com.br/</x:v>
+      </x:c>
+      <x:c r="J12" s="52" t="str">
+        <x:v>https://www.instagram.com/emerson.honda</x:v>
+      </x:c>
+      <x:c r="K12" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L12" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M12" s="52" t="str">
+        <x:v>Número/WhatsApp divulgado na bio/link público do próprio perfil; não validado pela empresa.. Site oficial Honda; lista Arapiraca, Maceió e União dos Palmares (3 lojas em AL). LinkedIn corporativo informa vínculo com Pernambuco Motos e outras unidades do grupo, mas validar se a prospecção será pela empresa local ou grupo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="56" customHeight="1">
+      <x:c r="A13" s="52" t="str">
+        <x:v>Jefferson Furstenau</x:v>
+      </x:c>
+      <x:c r="B13" s="52" t="str">
+        <x:v>@jefferson.sunmotors</x:v>
+      </x:c>
+      <x:c r="C13" s="52" t="str">
+        <x:v>Kia Sun Motors / Suzuki Sun Motors</x:v>
+      </x:c>
+      <x:c r="D13" s="52" t="str">
+        <x:v>kiasunmotors.com.br</x:v>
+      </x:c>
+      <x:c r="E13" s="52" t="str">
+        <x:v>Empresário / profissional automotivo</x:v>
+      </x:c>
+      <x:c r="F13" s="52" t="str"/>
+      <x:c r="G13" s="52" t="str"/>
+      <x:c r="H13" s="52" t="str">
+        <x:v>(51) 3382-1600 — site oficial/Kia</x:v>
+      </x:c>
+      <x:c r="I13" s="52" t="str">
+        <x:v>https://www.kiasunmotors.com.br/</x:v>
+      </x:c>
+      <x:c r="J13" s="52" t="str">
+        <x:v>https://www.instagram.com/jefferson.sunmotors</x:v>
+      </x:c>
+      <x:c r="K13" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L13" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M13" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Site oficial Kia Sun Motors em Porto Alegre; página oficial lista loja e contatos. Perfil menciona também Suzuki Sun Motors, relação/porte não confirmados.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="56" customHeight="1">
+      <x:c r="A14" s="52" t="str">
+        <x:v>Bruno Bettéro</x:v>
+      </x:c>
+      <x:c r="B14" s="52" t="str">
+        <x:v>@brunobettero</x:v>
+      </x:c>
+      <x:c r="C14" s="52" t="str">
+        <x:v>Concessionária não identificada na bio</x:v>
+      </x:c>
+      <x:c r="D14" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="E14" s="52" t="str">
+        <x:v>Gestor de Concessionária</x:v>
+      </x:c>
+      <x:c r="F14" s="52" t="str"/>
+      <x:c r="G14" s="52" t="str"/>
+      <x:c r="H14" s="52" t="str"/>
+      <x:c r="I14" s="52" t="str">
+        <x:v>https://alagoasmotos.com.br/</x:v>
+      </x:c>
+      <x:c r="J14" s="52" t="str">
+        <x:v>https://www.instagram.com/brunobettero</x:v>
+      </x:c>
+      <x:c r="K14" s="52" t="str">
+        <x:v>Domínio confirmado; vínculo da pessoa apoiado por fonte pública nominal</x:v>
+      </x:c>
+      <x:c r="L14" s="52" t="str">
+        <x:v>Página pública corporativa da Alagoas Motos lista Bruno Bettéro como gerente comercial; domínio confirmado apesar de a bio não citar empregador.</x:v>
+      </x:c>
+      <x:c r="M14" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Página corporativa/política pública da Alagoas Motos identifica Bruno Bettéro como gerente comercial; empresa/domínio confirmados por essa fonte nominal.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="56" customHeight="1">
+      <x:c r="A15" s="52" t="str">
+        <x:v>Gesivam Lopes</x:v>
+      </x:c>
+      <x:c r="B15" s="52" t="str">
+        <x:v>@gesivamlopes</x:v>
+      </x:c>
+      <x:c r="C15" s="52" t="str">
+        <x:v>Primavia Fiat</x:v>
+      </x:c>
+      <x:c r="D15" s="52" t="str">
+        <x:v>primaviafiat.com.br; grupoprimavia.com.br (grupo)</x:v>
+      </x:c>
+      <x:c r="E15" s="52" t="str">
+        <x:v>Gerente de Vendas</x:v>
+      </x:c>
+      <x:c r="F15" s="52" t="str"/>
+      <x:c r="G15" s="52" t="str">
+        <x:v>5561996665425</x:v>
+      </x:c>
+      <x:c r="H15" s="52" t="str"/>
+      <x:c r="I15" s="52" t="str">
+        <x:v>https://primaviafiat.com.br/</x:v>
+      </x:c>
+      <x:c r="J15" s="52" t="str">
+        <x:v>https://www.instagram.com/gesivamlopes</x:v>
+      </x:c>
+      <x:c r="K15" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L15" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M15" s="52" t="str">
+        <x:v>Número/WhatsApp divulgado na bio/link público do próprio perfil; não validado pela empresa.. Site oficial da concessionária Primavia Fiat e site institucional do grupo. Bio do lead declara Gerente de Vendas | Primavia Fiat; número de WhatsApp consta no link pessoal informado.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="56" customHeight="1">
+      <x:c r="A16" s="52" t="str">
+        <x:v>Keyanny</x:v>
+      </x:c>
+      <x:c r="B16" s="52" t="str">
+        <x:v>@keyannyalves</x:v>
+      </x:c>
+      <x:c r="C16" s="52" t="str">
+        <x:v>Original Yamaha</x:v>
+      </x:c>
+      <x:c r="D16" s="52" t="str">
+        <x:v>yamahaoriginal.com.br; originalautos.com.br (grupo)</x:v>
+      </x:c>
+      <x:c r="E16" s="52" t="str">
+        <x:v>Gerente</x:v>
+      </x:c>
+      <x:c r="F16" s="52" t="str"/>
+      <x:c r="G16" s="52" t="str"/>
+      <x:c r="H16" s="52" t="str"/>
+      <x:c r="I16" s="52" t="str">
+        <x:v>https://yamahaoriginal.com.br/</x:v>
+      </x:c>
+      <x:c r="J16" s="52" t="str">
+        <x:v>https://www.instagram.com/keyannyalves</x:v>
+      </x:c>
+      <x:c r="K16" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L16" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M16" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Site oficial Original Yamaha e site institucional Original Autos. Perfil correspondente/empregador não verificado nominalmente em fonte corporativa.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="56" customHeight="1">
+      <x:c r="A17" s="52" t="str">
+        <x:v>Reinaldo R. Cardoso | Conteúdo Automotivo</x:v>
+      </x:c>
+      <x:c r="B17" s="52" t="str">
+        <x:v>@reicardoso</x:v>
+      </x:c>
+      <x:c r="C17" s="52" t="str">
+        <x:v>Empresa não identificada na bio</x:v>
+      </x:c>
+      <x:c r="D17" s="52" t="str"/>
+      <x:c r="E17" s="52" t="str">
+        <x:v>Gerente Regional de Vendas</x:v>
+      </x:c>
+      <x:c r="F17" s="52" t="str"/>
+      <x:c r="G17" s="52" t="str"/>
+      <x:c r="H17" s="52" t="str"/>
+      <x:c r="I17" s="52" t="str"/>
+      <x:c r="J17" s="52" t="str">
+        <x:v>https://www.instagram.com/reicardoso</x:v>
+      </x:c>
+      <x:c r="K17" s="52" t="str">
+        <x:v>Sem domínio de empregador confirmado</x:v>
+      </x:c>
+      <x:c r="L17" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M17" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Empresa não identificável pelo nome/URL disponíveis no registro. Precisa pedir empregador/unidade ao lead antes de procurar canais corporativos.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="56" customHeight="1">
+      <x:c r="A18" s="52" t="str">
+        <x:v>Junior Mendes</x:v>
+      </x:c>
+      <x:c r="B18" s="52" t="str">
+        <x:v>@juniormendes___</x:v>
+      </x:c>
+      <x:c r="C18" s="52" t="str">
+        <x:v>Original São Luís</x:v>
+      </x:c>
+      <x:c r="D18" s="52" t="str">
+        <x:v>originalautos.com.br</x:v>
+      </x:c>
+      <x:c r="E18" s="52" t="str">
+        <x:v>Gerente Comercial</x:v>
+      </x:c>
+      <x:c r="F18" s="52" t="str"/>
+      <x:c r="G18" s="52" t="str"/>
+      <x:c r="H18" s="52" t="str"/>
+      <x:c r="I18" s="52" t="str">
+        <x:v>https://www.originalautos.com.br/empresa/original-autos</x:v>
+      </x:c>
+      <x:c r="J18" s="52" t="str">
+        <x:v>https://www.instagram.com/juniormendes___</x:v>
+      </x:c>
+      <x:c r="K18" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L18" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M18" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Site oficial Original Autos; empresa informa 13 lojas no Maranhão, incluindo várias marcas autorizadas. Conta tem fit de escala aparente; confirmar marca/unidade e vínculo atual da pessoa.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="56" customHeight="1">
+      <x:c r="A19" s="52" t="str">
+        <x:v>Ana Angélica</x:v>
+      </x:c>
+      <x:c r="B19" s="52" t="str">
+        <x:v>@angelicaomena</x:v>
+      </x:c>
+      <x:c r="C19" s="52" t="str">
+        <x:v>Grupo Gama</x:v>
+      </x:c>
+      <x:c r="D19" s="52" t="str">
+        <x:v>grupogama.com.br</x:v>
+      </x:c>
+      <x:c r="E19" s="52" t="str">
+        <x:v>Gerente Comercial</x:v>
+      </x:c>
+      <x:c r="F19" s="52" t="str"/>
+      <x:c r="G19" s="52" t="str"/>
+      <x:c r="H19" s="52" t="str"/>
+      <x:c r="I19" s="52" t="str">
+        <x:v>https://www.grupogama.com.br/concessionarias-do-grupo</x:v>
+      </x:c>
+      <x:c r="J19" s="52" t="str">
+        <x:v>https://www.instagram.com/angelicaomena</x:v>
+      </x:c>
+      <x:c r="K19" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L19" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M19" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Site oficial lista várias concessionárias/marcas e atuação em mais de um estado; posição de Ana Angélica no grupo não foi achada em página corporativa.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="56" customHeight="1">
+      <x:c r="A20" s="52" t="str">
+        <x:v>Gessiane Nina| Original Caoa Chery</x:v>
+      </x:c>
+      <x:c r="B20" s="52" t="str">
+        <x:v>@gessiane.nina</x:v>
+      </x:c>
+      <x:c r="C20" s="52" t="str">
+        <x:v>CAOA Chery Original São Luís</x:v>
+      </x:c>
+      <x:c r="D20" s="52" t="str">
+        <x:v>originalautos.com.br</x:v>
+      </x:c>
+      <x:c r="E20" s="52" t="str">
+        <x:v>Gerente Comercial</x:v>
+      </x:c>
+      <x:c r="F20" s="52" t="str"/>
+      <x:c r="G20" s="52" t="str"/>
+      <x:c r="H20" s="52" t="str"/>
+      <x:c r="I20" s="52" t="str">
+        <x:v>https://www.originalautos.com.br/empresa/original-autos</x:v>
+      </x:c>
+      <x:c r="J20" s="52" t="str">
+        <x:v>https://www.instagram.com/gessiane.nina</x:v>
+      </x:c>
+      <x:c r="K20" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L20" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M20" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Site oficial Original Autos; empresa informa 13 lojas no Maranhão, incluindo várias marcas autorizadas. Conta tem fit de escala aparente; confirmar marca/unidade e vínculo atual da pessoa.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="56" customHeight="1">
+      <x:c r="A21" s="52" t="str">
+        <x:v>Leandro Guimarães</x:v>
+      </x:c>
+      <x:c r="B21" s="52" t="str">
+        <x:v>@leandroguimaraesal</x:v>
+      </x:c>
+      <x:c r="C21" s="52" t="str">
+        <x:v>Alagoas Motos</x:v>
+      </x:c>
+      <x:c r="D21" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="E21" s="52" t="str">
+        <x:v>Gerente Comercial</x:v>
+      </x:c>
+      <x:c r="F21" s="52" t="str"/>
+      <x:c r="G21" s="52" t="str"/>
+      <x:c r="H21" s="52" t="str">
+        <x:v>(82) 3539-8605; WhatsApp geral (82) 99996-0571 — site oficial</x:v>
+      </x:c>
+      <x:c r="I21" s="52" t="str">
+        <x:v>https://alagoasmotos.com.br/</x:v>
+      </x:c>
+      <x:c r="J21" s="52" t="str">
+        <x:v>https://www.instagram.com/leandroguimaraesal</x:v>
+      </x:c>
+      <x:c r="K21" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L21" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M21" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Site oficial Honda; lista Arapiraca, Maceió e União dos Palmares (3 lojas em AL). LinkedIn corporativo informa vínculo com Pernambuco Motos e outras unidades do grupo, mas validar se a prospecção será pela empresa local ou grupo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="56" customHeight="1">
+      <x:c r="A22" s="52" t="str">
+        <x:v>Wallas Oliveira</x:v>
+      </x:c>
+      <x:c r="B22" s="52" t="str">
+        <x:v>@wallasoliveira</x:v>
+      </x:c>
+      <x:c r="C22" s="52" t="str">
+        <x:v>Your Best Car BSB</x:v>
+      </x:c>
+      <x:c r="D22" s="52" t="str"/>
+      <x:c r="E22" s="52" t="str">
+        <x:v>Head Comercial</x:v>
+      </x:c>
+      <x:c r="F22" s="52" t="str"/>
+      <x:c r="G22" s="52" t="str"/>
+      <x:c r="H22" s="52" t="str"/>
+      <x:c r="I22" s="52" t="str"/>
+      <x:c r="J22" s="52" t="str">
+        <x:v>https://www.instagram.com/wallasoliveira</x:v>
+      </x:c>
+      <x:c r="K22" s="52" t="str">
+        <x:v>Sem domínio de empregador confirmado</x:v>
+      </x:c>
+      <x:c r="L22" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M22" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Não localizei domínio oficial inequívoco para a empresa exata; resultados homônimos/contas de seminovos não bastam para atribuição.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="56" customHeight="1">
+      <x:c r="A23" s="52" t="str">
+        <x:v>Lucas Abreu /Carros Seminovos</x:v>
+      </x:c>
+      <x:c r="B23" s="52" t="str">
+        <x:v>@lucas.babreu</x:v>
+      </x:c>
+      <x:c r="C23" s="52" t="str">
+        <x:v>Original Autos</x:v>
+      </x:c>
+      <x:c r="D23" s="52" t="str">
+        <x:v>originalautos.com.br</x:v>
+      </x:c>
+      <x:c r="E23" s="52" t="str">
+        <x:v>Gestor Comercial</x:v>
+      </x:c>
+      <x:c r="F23" s="52" t="str"/>
+      <x:c r="G23" s="52" t="str"/>
+      <x:c r="H23" s="52" t="str"/>
+      <x:c r="I23" s="52" t="str">
+        <x:v>https://www.originalautos.com.br/empresa/original-autos</x:v>
+      </x:c>
+      <x:c r="J23" s="52" t="str">
+        <x:v>https://www.instagram.com/lucas.babreu</x:v>
+      </x:c>
+      <x:c r="K23" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L23" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M23" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Site institucional confirma a rede; o perfil individual não foi encontrado entre os nomes publicados pela empresa.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="56" customHeight="1">
+      <x:c r="A24" s="52" t="str">
+        <x:v>Soljane Mendes</x:v>
+      </x:c>
+      <x:c r="B24" s="52" t="str">
+        <x:v>@antoniasolijane</x:v>
+      </x:c>
+      <x:c r="C24" s="52" t="str">
+        <x:v>Renault Original São Luís</x:v>
+      </x:c>
+      <x:c r="D24" s="52" t="str">
+        <x:v>originalautos.com.br</x:v>
+      </x:c>
+      <x:c r="E24" s="52" t="str">
+        <x:v>Gerente de Pós-Vendas</x:v>
+      </x:c>
+      <x:c r="F24" s="52" t="str"/>
+      <x:c r="G24" s="52" t="str"/>
+      <x:c r="H24" s="52" t="str"/>
+      <x:c r="I24" s="52" t="str">
+        <x:v>https://www.originalautos.com.br/empresa/original-autos</x:v>
+      </x:c>
+      <x:c r="J24" s="52" t="str">
+        <x:v>https://www.instagram.com/antoniasolijane</x:v>
+      </x:c>
+      <x:c r="K24" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L24" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M24" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Site oficial Original Autos; empresa informa 13 lojas no Maranhão, incluindo várias marcas autorizadas. Conta tem fit de escala aparente; confirmar marca/unidade e vínculo atual da pessoa.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="56" customHeight="1">
+      <x:c r="A25" s="52" t="str">
+        <x:v>Mineiro da Honda | Consórcio em Arapiraca</x:v>
+      </x:c>
+      <x:c r="B25" s="52" t="str">
+        <x:v>@izael_doconsorcio</x:v>
+      </x:c>
+      <x:c r="C25" s="52" t="str">
+        <x:v>Alagoas Motos</x:v>
+      </x:c>
+      <x:c r="D25" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="E25" s="52" t="str">
+        <x:v>Supervisor de Vendas</x:v>
+      </x:c>
+      <x:c r="F25" s="52" t="str"/>
+      <x:c r="G25" s="52" t="str">
+        <x:v>558220013162</x:v>
+      </x:c>
+      <x:c r="H25" s="52" t="str">
+        <x:v>(82) 3539-8605; WhatsApp geral (82) 99996-0571 — site oficial</x:v>
+      </x:c>
+      <x:c r="I25" s="52" t="str">
+        <x:v>https://alagoasmotos.com.br/</x:v>
+      </x:c>
+      <x:c r="J25" s="52" t="str">
+        <x:v>https://www.instagram.com/izael_doconsorcio</x:v>
+      </x:c>
+      <x:c r="K25" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L25" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M25" s="52" t="str">
+        <x:v>Número/WhatsApp divulgado na bio/link público do próprio perfil; não validado pela empresa.. Site oficial Honda; lista Arapiraca, Maceió e União dos Palmares (3 lojas em AL). LinkedIn corporativo informa vínculo com Pernambuco Motos e outras unidades do grupo, mas validar se a prospecção será pela empresa local ou grupo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="56" customHeight="1">
+      <x:c r="A26" s="52" t="str">
+        <x:v>FAGNÉ </x:v>
+      </x:c>
+      <x:c r="B26" s="52" t="str">
+        <x:v>@fagnerdahonda</x:v>
+      </x:c>
+      <x:c r="C26" s="52" t="str">
+        <x:v>Alagoas Motos</x:v>
+      </x:c>
+      <x:c r="D26" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="E26" s="52" t="str">
+        <x:v>Supervisor de Vendas</x:v>
+      </x:c>
+      <x:c r="F26" s="52" t="str"/>
+      <x:c r="G26" s="52" t="str">
+        <x:v>5582993424355</x:v>
+      </x:c>
+      <x:c r="H26" s="52" t="str">
+        <x:v>(82) 3539-8605; WhatsApp geral (82) 99996-0571 — site oficial</x:v>
+      </x:c>
+      <x:c r="I26" s="52" t="str">
+        <x:v>https://alagoasmotos.com.br/</x:v>
+      </x:c>
+      <x:c r="J26" s="52" t="str">
+        <x:v>https://www.instagram.com/fagnerdahonda</x:v>
+      </x:c>
+      <x:c r="K26" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L26" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M26" s="52" t="str">
+        <x:v>Número/WhatsApp divulgado na bio/link público do próprio perfil; não validado pela empresa.. Site oficial Honda; lista Arapiraca, Maceió e União dos Palmares (3 lojas em AL). LinkedIn corporativo informa vínculo com Pernambuco Motos e outras unidades do grupo, mas validar se a prospecção será pela empresa local ou grupo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="56" customHeight="1">
+      <x:c r="A27" s="52" t="str">
+        <x:v>Klebson Wesley | Consórcio Honda</x:v>
+      </x:c>
+      <x:c r="B27" s="52" t="str">
+        <x:v>@klebson_honda</x:v>
+      </x:c>
+      <x:c r="C27" s="52" t="str">
+        <x:v>Alagoas Motos</x:v>
+      </x:c>
+      <x:c r="D27" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="E27" s="52" t="str">
+        <x:v>Supervisor de Vendas</x:v>
+      </x:c>
+      <x:c r="F27" s="52" t="str"/>
+      <x:c r="G27" s="52" t="str">
+        <x:v>5582999580622</x:v>
+      </x:c>
+      <x:c r="H27" s="52" t="str">
+        <x:v>(82) 3539-8605; WhatsApp geral (82) 99996-0571 — site oficial</x:v>
+      </x:c>
+      <x:c r="I27" s="52" t="str">
+        <x:v>https://alagoasmotos.com.br/</x:v>
+      </x:c>
+      <x:c r="J27" s="52" t="str">
+        <x:v>https://www.instagram.com/klebson_honda</x:v>
+      </x:c>
+      <x:c r="K27" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L27" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M27" s="52" t="str">
+        <x:v>Número profissional publicamente associado ao perfil em fonte social; valide antes do contato.. Site oficial Honda; lista Arapiraca, Maceió e União dos Palmares (3 lojas em AL). LinkedIn corporativo informa vínculo com Pernambuco Motos e outras unidades do grupo, mas validar se a prospecção será pela empresa local ou grupo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="56" customHeight="1">
+      <x:c r="A28" s="52" t="str">
+        <x:v>CRYS DA HONDA / CONSÓRCIO HONDA 🏆🥇🙏</x:v>
+      </x:c>
+      <x:c r="B28" s="52" t="str">
+        <x:v>@crys_da_honda</x:v>
+      </x:c>
+      <x:c r="C28" s="52" t="str">
+        <x:v>Alagoas Motos</x:v>
+      </x:c>
+      <x:c r="D28" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="E28" s="52" t="str">
+        <x:v>Supervisora de Vendas</x:v>
+      </x:c>
+      <x:c r="F28" s="52" t="str"/>
+      <x:c r="G28" s="52" t="str">
+        <x:v>5582993262015</x:v>
+      </x:c>
+      <x:c r="H28" s="52" t="str">
+        <x:v>(82) 3539-8605; WhatsApp geral (82) 99996-0571 — site oficial</x:v>
+      </x:c>
+      <x:c r="I28" s="52" t="str">
+        <x:v>https://alagoasmotos.com.br/</x:v>
+      </x:c>
+      <x:c r="J28" s="52" t="str">
+        <x:v>https://www.instagram.com/crys_da_honda</x:v>
+      </x:c>
+      <x:c r="K28" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L28" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M28" s="52" t="str">
+        <x:v>Número profissional publicamente associado ao perfil em fonte social; valide antes do contato.. Site oficial Honda; lista Arapiraca, Maceió e União dos Palmares (3 lojas em AL). LinkedIn corporativo informa vínculo com Pernambuco Motos e outras unidades do grupo, mas validar se a prospecção será pela empresa local ou grupo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="56" customHeight="1">
+      <x:c r="A29" s="52" t="str">
+        <x:v>GSerejo 🏅</x:v>
+      </x:c>
+      <x:c r="B29" s="52" t="str">
+        <x:v>@lennyserejo</x:v>
+      </x:c>
+      <x:c r="C29" s="52" t="str">
+        <x:v>Original São Luís</x:v>
+      </x:c>
+      <x:c r="D29" s="52" t="str">
+        <x:v>originalautos.com.br</x:v>
+      </x:c>
+      <x:c r="E29" s="52" t="str">
+        <x:v>Especialista em Pós-Vendas</x:v>
+      </x:c>
+      <x:c r="F29" s="52" t="str"/>
+      <x:c r="G29" s="52" t="str"/>
+      <x:c r="H29" s="52" t="str"/>
+      <x:c r="I29" s="52" t="str">
+        <x:v>https://www.originalautos.com.br/empresa/original-autos</x:v>
+      </x:c>
+      <x:c r="J29" s="52" t="str">
+        <x:v>https://www.instagram.com/lennyserejo</x:v>
+      </x:c>
+      <x:c r="K29" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L29" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M29" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Site oficial Original Autos; empresa informa 13 lojas no Maranhão, incluindo várias marcas autorizadas. Conta tem fit de escala aparente; confirmar marca/unidade e vínculo atual da pessoa.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="56" customHeight="1">
+      <x:c r="A30" s="52" t="str">
+        <x:v>Gelison Ramos | Consórcio Honda Brasil 🇧🇷</x:v>
+      </x:c>
+      <x:c r="B30" s="52" t="str">
+        <x:v>@gelisonhonda</x:v>
+      </x:c>
+      <x:c r="C30" s="52" t="str">
+        <x:v>Alagoas Motos</x:v>
+      </x:c>
+      <x:c r="D30" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="E30" s="52" t="str">
+        <x:v>Supervisor de Vendas</x:v>
+      </x:c>
+      <x:c r="F30" s="52" t="str"/>
+      <x:c r="G30" s="52" t="str"/>
+      <x:c r="H30" s="52" t="str">
+        <x:v>(82) 3539-8605; WhatsApp geral (82) 99996-0571 — site oficial</x:v>
+      </x:c>
+      <x:c r="I30" s="52" t="str">
+        <x:v>https://alagoasmotos.com.br/</x:v>
+      </x:c>
+      <x:c r="J30" s="52" t="str">
+        <x:v>https://www.instagram.com/gelisonhonda</x:v>
+      </x:c>
+      <x:c r="K30" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L30" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M30" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Site oficial Honda; lista Arapiraca, Maceió e União dos Palmares (3 lojas em AL). LinkedIn corporativo informa vínculo com Pernambuco Motos e outras unidades do grupo, mas validar se a prospecção será pela empresa local ou grupo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="56" customHeight="1">
+      <x:c r="A31" s="52" t="str">
+        <x:v>Adrielle Bezerra</x:v>
+      </x:c>
+      <x:c r="B31" s="52" t="str">
+        <x:v>@adriellehondaa</x:v>
+      </x:c>
+      <x:c r="C31" s="52" t="str">
+        <x:v>Alagoas Motos</x:v>
+      </x:c>
+      <x:c r="D31" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="E31" s="52" t="str">
+        <x:v>Vendedora de Financiamento</x:v>
+      </x:c>
+      <x:c r="F31" s="52" t="str"/>
+      <x:c r="G31" s="52" t="str">
+        <x:v>5582996416647</x:v>
+      </x:c>
+      <x:c r="H31" s="52" t="str">
+        <x:v>(82) 3539-8605; WhatsApp geral (82) 99996-0571 — site oficial</x:v>
+      </x:c>
+      <x:c r="I31" s="52" t="str">
+        <x:v>https://alagoasmotos.com.br/</x:v>
+      </x:c>
+      <x:c r="J31" s="52" t="str">
+        <x:v>https://www.instagram.com/adriellehondaa</x:v>
+      </x:c>
+      <x:c r="K31" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L31" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M31" s="52" t="str">
+        <x:v>Número/WhatsApp divulgado na bio/link público do próprio perfil; não validado pela empresa.. Site oficial Honda; lista Arapiraca, Maceió e União dos Palmares (3 lojas em AL). LinkedIn corporativo informa vínculo com Pernambuco Motos e outras unidades do grupo, mas validar se a prospecção será pela empresa local ou grupo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="56" customHeight="1">
+      <x:c r="A32" s="52" t="str">
+        <x:v>Jô Vieira - 🚘Q Vendas🚘</x:v>
+      </x:c>
+      <x:c r="B32" s="52" t="str">
+        <x:v>@jovieira_qvendas</x:v>
+      </x:c>
+      <x:c r="C32" s="52" t="str">
+        <x:v>Q Vendas</x:v>
+      </x:c>
+      <x:c r="D32" s="52" t="str">
+        <x:v>quevendas.com.br</x:v>
+      </x:c>
+      <x:c r="E32" s="52" t="str">
+        <x:v>Consultora de Vendas</x:v>
+      </x:c>
+      <x:c r="F32" s="52" t="str"/>
+      <x:c r="G32" s="52" t="str">
+        <x:v>55964722870</x:v>
+      </x:c>
+      <x:c r="H32" s="52" t="str">
+        <x:v>(21) 2137-1252; (21) 97436-4644 — site oficial</x:v>
+      </x:c>
+      <x:c r="I32" s="52" t="str">
+        <x:v>https://www.quevendas.com.br/</x:v>
+      </x:c>
+      <x:c r="J32" s="52" t="str">
+        <x:v>https://www.instagram.com/jovieira_qvendas</x:v>
+      </x:c>
+      <x:c r="K32" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L32" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M32" s="52" t="str">
+        <x:v>Número/WhatsApp divulgado na bio/link público do próprio perfil; não validado pela empresa.. Site oficial confirma loja de compra/venda multimarcas no Rio de Janeiro; não é evidência de concessionária autorizada monomarca.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="56" customHeight="1">
+      <x:c r="A33" s="52" t="str">
+        <x:v>Elaine Brumati</x:v>
+      </x:c>
+      <x:c r="B33" s="52" t="str">
+        <x:v>@elainebrumati</x:v>
+      </x:c>
+      <x:c r="C33" s="52" t="str">
+        <x:v>Honda</x:v>
+      </x:c>
+      <x:c r="D33" s="52" t="str"/>
+      <x:c r="E33" s="52" t="str">
+        <x:v>Especialista em Contemplação Honda</x:v>
+      </x:c>
+      <x:c r="F33" s="52" t="str"/>
+      <x:c r="G33" s="52" t="str">
+        <x:v>5565999057068</x:v>
+      </x:c>
+      <x:c r="H33" s="52" t="str"/>
+      <x:c r="I33" s="52" t="str"/>
+      <x:c r="J33" s="52" t="str">
+        <x:v>https://www.instagram.com/elainebrumati</x:v>
+      </x:c>
+      <x:c r="K33" s="52" t="str">
+        <x:v>Sem domínio de empregador confirmado</x:v>
+      </x:c>
+      <x:c r="L33" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M33" s="52" t="str">
+        <x:v>Número/WhatsApp divulgado na bio/link público do próprio perfil; não validado pela empresa.. “Honda” é marca/produto e não identifica concessionária empregadora. Perfis ligados à Alagoas Motos estão associados ao respectivo domínio quando explícito; nos demais, sem domínio de empresa atribuído.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="56" customHeight="1">
+      <x:c r="A34" s="52" t="str">
+        <x:v>Weryka Samara/Consórcio Honda</x:v>
+      </x:c>
+      <x:c r="B34" s="52" t="str">
+        <x:v>@werykasamara_honda</x:v>
+      </x:c>
+      <x:c r="C34" s="52" t="str">
+        <x:v>Honda</x:v>
+      </x:c>
+      <x:c r="D34" s="52" t="str"/>
+      <x:c r="E34" s="52" t="str">
+        <x:v>Especialista Honda</x:v>
+      </x:c>
+      <x:c r="F34" s="52" t="str"/>
+      <x:c r="G34" s="52" t="str">
+        <x:v>(82)99609-1225</x:v>
+      </x:c>
+      <x:c r="H34" s="52" t="str"/>
+      <x:c r="I34" s="52" t="str"/>
+      <x:c r="J34" s="52" t="str">
+        <x:v>https://www.instagram.com/werykasamara_honda</x:v>
+      </x:c>
+      <x:c r="K34" s="52" t="str">
+        <x:v>Sem domínio de empregador confirmado</x:v>
+      </x:c>
+      <x:c r="L34" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M34" s="52" t="str">
+        <x:v>Número/WhatsApp divulgado na bio/link público do próprio perfil; não validado pela empresa.. “Honda” é marca/produto e não identifica concessionária empregadora. Perfis ligados à Alagoas Motos estão associados ao respectivo domínio quando explícito; nos demais, sem domínio de empresa atribuído.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="56" customHeight="1">
+      <x:c r="A35" s="52" t="str">
+        <x:v>Paulo Borba</x:v>
+      </x:c>
+      <x:c r="B35" s="52" t="str">
+        <x:v>@borba.nissan</x:v>
+      </x:c>
+      <x:c r="C35" s="52" t="str">
+        <x:v>Nissan / Geely em Lages</x:v>
+      </x:c>
+      <x:c r="D35" s="52" t="str">
+        <x:v>drsulnissan.com.br (unidade Nissan Lages; vínculo apoiado pela bio)</x:v>
+      </x:c>
+      <x:c r="E35" s="52" t="str">
+        <x:v>Consultor / vendedor automotivo</x:v>
+      </x:c>
+      <x:c r="F35" s="52" t="str"/>
+      <x:c r="G35" s="52" t="str">
+        <x:v>5548991914093</x:v>
+      </x:c>
+      <x:c r="H35" s="52" t="str"/>
+      <x:c r="I35" s="52" t="str">
+        <x:v>https://www.drsulnissan.com.br/drsul-nissan-lages-sc/contato/fale-conosco</x:v>
+      </x:c>
+      <x:c r="J35" s="52" t="str">
+        <x:v>https://www.instagram.com/borba.nissan</x:v>
+      </x:c>
+      <x:c r="K35" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L35" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M35" s="52" t="str">
+        <x:v>Número/WhatsApp divulgado na bio/link público do próprio perfil; não validado pela empresa.. Site oficial da DRSUL Nissan Lages; perfil declara Nissan/Geely e Lages. Telefone no perfil é WhatsApp profissional publicado pelo próprio lead.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="56" customHeight="1">
+      <x:c r="A36" s="52" t="str">
+        <x:v>Wendell Brandão | Consultor Honda 🏍️</x:v>
+      </x:c>
+      <x:c r="B36" s="52" t="str">
+        <x:v>@wendellhondaa</x:v>
+      </x:c>
+      <x:c r="C36" s="52" t="str">
+        <x:v>Honda</x:v>
+      </x:c>
+      <x:c r="D36" s="52" t="str"/>
+      <x:c r="E36" s="52" t="str">
+        <x:v>Consultor Honda</x:v>
+      </x:c>
+      <x:c r="F36" s="52" t="str"/>
+      <x:c r="G36" s="52" t="str">
+        <x:v>8299581244</x:v>
+      </x:c>
+      <x:c r="H36" s="52" t="str"/>
+      <x:c r="I36" s="52" t="str"/>
+      <x:c r="J36" s="52" t="str">
+        <x:v>https://www.instagram.com/wendellhondaa</x:v>
+      </x:c>
+      <x:c r="K36" s="52" t="str">
+        <x:v>Sem domínio de empregador confirmado</x:v>
+      </x:c>
+      <x:c r="L36" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M36" s="52" t="str">
+        <x:v>Número/WhatsApp divulgado na bio/link público do próprio perfil; não validado pela empresa.. “Honda” é marca/produto e não identifica concessionária empregadora. Perfis ligados à Alagoas Motos estão associados ao respectivo domínio quando explícito; nos demais, sem domínio de empresa atribuído.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="56" customHeight="1">
+      <x:c r="A37" s="52" t="str">
+        <x:v>Bruno Fernando</x:v>
+      </x:c>
+      <x:c r="B37" s="52" t="str">
+        <x:v>@bruno.fernando.fiatslz</x:v>
+      </x:c>
+      <x:c r="C37" s="52" t="str">
+        <x:v>Fiat Original São Luís</x:v>
+      </x:c>
+      <x:c r="D37" s="52" t="str">
+        <x:v>originalautos.com.br</x:v>
+      </x:c>
+      <x:c r="E37" s="52" t="str">
+        <x:v>Executivo de Vendas</x:v>
+      </x:c>
+      <x:c r="F37" s="52" t="str"/>
+      <x:c r="G37" s="52" t="str">
+        <x:v>5598981205421</x:v>
+      </x:c>
+      <x:c r="H37" s="52" t="str"/>
+      <x:c r="I37" s="52" t="str">
+        <x:v>https://www.originalautos.com.br/empresa/original-autos</x:v>
+      </x:c>
+      <x:c r="J37" s="52" t="str">
+        <x:v>https://www.instagram.com/bruno.fernando.fiatslz</x:v>
+      </x:c>
+      <x:c r="K37" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L37" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M37" s="52" t="str">
+        <x:v>Número/WhatsApp divulgado na bio/link público do próprio perfil; não validado pela empresa.. Site oficial Original Autos; empresa informa 13 lojas no Maranhão, incluindo várias marcas autorizadas. Conta tem fit de escala aparente; confirmar marca/unidade e vínculo atual da pessoa.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="56" customHeight="1">
+      <x:c r="A38" s="52" t="str">
+        <x:v>Eduardo Pitta Pontual</x:v>
+      </x:c>
+      <x:c r="B38" s="52" t="str">
+        <x:v>@eduardopittapontual</x:v>
+      </x:c>
+      <x:c r="C38" s="52" t="str">
+        <x:v>Italiana Automóveis</x:v>
+      </x:c>
+      <x:c r="D38" s="52" t="str">
+        <x:v>italiana.com.br</x:v>
+      </x:c>
+      <x:c r="E38" s="52" t="str">
+        <x:v>Profissional de concessionária</x:v>
+      </x:c>
+      <x:c r="F38" s="52" t="str"/>
+      <x:c r="G38" s="52" t="str"/>
+      <x:c r="H38" s="52" t="str">
+        <x:v>Vendas Recife: (81) 2121-1100; WhatsApp corporativo: (81) 98258-1100 — site oficial</x:v>
+      </x:c>
+      <x:c r="I38" s="52" t="str">
+        <x:v>https://www.italiana.com.br/</x:v>
+      </x:c>
+      <x:c r="J38" s="52" t="str">
+        <x:v>https://www.instagram.com/eduardopittapontual</x:v>
+      </x:c>
+      <x:c r="K38" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L38" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M38" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Site oficial do Grupo Italiana confirma empresa; site Fiat Italiana lista 3 lojas (Recife Imbiribeira, Caxangá e Caruaru). Canal geral de vendas disponível no site.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="56" customHeight="1">
+      <x:c r="A39" s="52" t="str">
+        <x:v>Alexandre Hoffmann</x:v>
+      </x:c>
+      <x:c r="B39" s="52" t="str">
+        <x:v>@ahoffmannveiculos</x:v>
+      </x:c>
+      <x:c r="C39" s="52" t="str">
+        <x:v>Hoffmann Veículos</x:v>
+      </x:c>
+      <x:c r="D39" s="52" t="str">
+        <x:v>ahoffmannveiculos.com</x:v>
+      </x:c>
+      <x:c r="E39" s="52" t="str">
+        <x:v>Profissional automotivo</x:v>
+      </x:c>
+      <x:c r="F39" s="52" t="str"/>
+      <x:c r="G39" s="52" t="str">
+        <x:v>(61) 99936-9991</x:v>
+      </x:c>
+      <x:c r="H39" s="52" t="str"/>
+      <x:c r="I39" s="52" t="str">
+        <x:v>https://www.ahoffmannveiculos.com/contato</x:v>
+      </x:c>
+      <x:c r="J39" s="52" t="str">
+        <x:v>https://www.instagram.com/ahoffmannveiculos</x:v>
+      </x:c>
+      <x:c r="K39" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L39" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M39" s="52" t="str">
+        <x:v>Número/WhatsApp divulgado na bio/link público do próprio perfil; não validado pela empresa.. Site oficial da empresa, mas telefone/e-mail são canais corporativos. Perfil é da empresa/lead, porém nenhum canal foi tratado como contato pessoal.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="56" customHeight="1">
+      <x:c r="A40" s="52" t="str">
+        <x:v>Luiz Henrique Tubarão</x:v>
+      </x:c>
+      <x:c r="B40" s="52" t="str">
+        <x:v>@luizhenriquetubarao</x:v>
+      </x:c>
+      <x:c r="C40" s="52" t="str">
+        <x:v>Grupo Euroaméricas</x:v>
+      </x:c>
+      <x:c r="D40" s="52" t="str">
+        <x:v>eurobarrafiat.com.br (loja Fiat do grupo)</x:v>
+      </x:c>
+      <x:c r="E40" s="52" t="str">
+        <x:v>Sales Manager</x:v>
+      </x:c>
+      <x:c r="F40" s="52" t="str"/>
+      <x:c r="G40" s="52" t="str"/>
+      <x:c r="H40" s="52" t="str"/>
+      <x:c r="I40" s="52" t="str">
+        <x:v>https://www.eurobarrafiat.com.br/politica-de-privacidade</x:v>
+      </x:c>
+      <x:c r="J40" s="52" t="str">
+        <x:v>https://www.instagram.com/luizhenriquetubarao</x:v>
+      </x:c>
+      <x:c r="K40" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L40" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M40" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Domínio oficial de concessionária do grupo. A bio de Luiz declara Sales Manager no Grupo Euroaméricas; WhatsApp pessoal foi encontrado em conteúdo público do próprio perfil.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="56" customHeight="1">
+      <x:c r="A41" s="52" t="str">
+        <x:v>ALEXANDRE | CONSÓRCIO HONDA</x:v>
+      </x:c>
+      <x:c r="B41" s="52" t="str">
+        <x:v>@alexandrechonda</x:v>
+      </x:c>
+      <x:c r="C41" s="52" t="str">
+        <x:v>Consórcio Honda</x:v>
+      </x:c>
+      <x:c r="D41" s="52" t="str"/>
+      <x:c r="E41" s="52" t="str">
+        <x:v>Especialista em Consórcio Honda</x:v>
+      </x:c>
+      <x:c r="F41" s="52" t="str"/>
+      <x:c r="G41" s="52" t="str"/>
+      <x:c r="H41" s="52" t="str"/>
+      <x:c r="I41" s="52" t="str"/>
+      <x:c r="J41" s="52" t="str">
+        <x:v>https://www.instagram.com/alexandrechonda</x:v>
+      </x:c>
+      <x:c r="K41" s="52" t="str">
+        <x:v>Sem domínio de empregador confirmado</x:v>
+      </x:c>
+      <x:c r="L41" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M41" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. “Honda” é marca/produto e não identifica concessionária empregadora. Perfis ligados à Alagoas Motos estão associados ao respectivo domínio quando explícito; nos demais, sem domínio de empresa atribuído.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="56" customHeight="1">
+      <x:c r="A42" s="52" t="str">
+        <x:v>Italo Antonio | Consórcio Honda | Moto 0KM 🏍️</x:v>
+      </x:c>
+      <x:c r="B42" s="52" t="str">
+        <x:v>@italodahonda082</x:v>
+      </x:c>
+      <x:c r="C42" s="52" t="str">
+        <x:v>Honda</x:v>
+      </x:c>
+      <x:c r="D42" s="52" t="str"/>
+      <x:c r="E42" s="52" t="str">
+        <x:v>Especialista em Consórcio Honda</x:v>
+      </x:c>
+      <x:c r="F42" s="52" t="str"/>
+      <x:c r="G42" s="52" t="str"/>
+      <x:c r="H42" s="52" t="str"/>
+      <x:c r="I42" s="52" t="str"/>
+      <x:c r="J42" s="52" t="str">
+        <x:v>https://www.instagram.com/italodahonda082</x:v>
+      </x:c>
+      <x:c r="K42" s="52" t="str">
+        <x:v>Sem domínio de empregador confirmado</x:v>
+      </x:c>
+      <x:c r="L42" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M42" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. “Honda” é marca/produto e não identifica concessionária empregadora. Perfis ligados à Alagoas Motos estão associados ao respectivo domínio quando explícito; nos demais, sem domínio de empresa atribuído.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="56" customHeight="1">
+      <x:c r="A43" s="52" t="str">
+        <x:v>Guilherme Caetano</x:v>
+      </x:c>
+      <x:c r="B43" s="52" t="str">
+        <x:v>@guilherme.honda1</x:v>
+      </x:c>
+      <x:c r="C43" s="52" t="str">
+        <x:v>Consórcio Honda</x:v>
+      </x:c>
+      <x:c r="D43" s="52" t="str"/>
+      <x:c r="E43" s="52" t="str">
+        <x:v>Especialista em Consórcio Honda</x:v>
+      </x:c>
+      <x:c r="F43" s="52" t="str"/>
+      <x:c r="G43" s="52" t="str"/>
+      <x:c r="H43" s="52" t="str"/>
+      <x:c r="I43" s="52" t="str"/>
+      <x:c r="J43" s="52" t="str">
+        <x:v>https://www.instagram.com/guilherme.honda1</x:v>
+      </x:c>
+      <x:c r="K43" s="52" t="str">
+        <x:v>Sem domínio de empregador confirmado</x:v>
+      </x:c>
+      <x:c r="L43" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M43" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. “Honda” é marca/produto e não identifica concessionária empregadora. Perfis ligados à Alagoas Motos estão associados ao respectivo domínio quando explícito; nos demais, sem domínio de empresa atribuído.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="56" customHeight="1">
+      <x:c r="A44" s="52" t="str">
+        <x:v>Karoll cavalcante | Honda</x:v>
+      </x:c>
+      <x:c r="B44" s="52" t="str">
+        <x:v>@karollhonda</x:v>
+      </x:c>
+      <x:c r="C44" s="52" t="str">
+        <x:v>Alagoas Motos</x:v>
+      </x:c>
+      <x:c r="D44" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="E44" s="52" t="str">
+        <x:v>Vendedora Web</x:v>
+      </x:c>
+      <x:c r="F44" s="52" t="str"/>
+      <x:c r="G44" s="52" t="str"/>
+      <x:c r="H44" s="52" t="str">
+        <x:v>(82) 3539-8605; WhatsApp geral (82) 99996-0571 — site oficial</x:v>
+      </x:c>
+      <x:c r="I44" s="52" t="str">
+        <x:v>https://alagoasmotos.com.br/</x:v>
+      </x:c>
+      <x:c r="J44" s="52" t="str">
+        <x:v>https://www.instagram.com/karollhonda</x:v>
+      </x:c>
+      <x:c r="K44" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L44" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M44" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Site oficial Honda; lista Arapiraca, Maceió e União dos Palmares (3 lojas em AL). LinkedIn corporativo informa vínculo com Pernambuco Motos e outras unidades do grupo, mas validar se a prospecção será pela empresa local ou grupo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="56" customHeight="1">
+      <x:c r="A45" s="52" t="str">
+        <x:v>Mayara da Honda</x:v>
+      </x:c>
+      <x:c r="B45" s="52" t="str">
+        <x:v>@mayaradahonda</x:v>
+      </x:c>
+      <x:c r="C45" s="52" t="str">
+        <x:v>Honda</x:v>
+      </x:c>
+      <x:c r="D45" s="52" t="str"/>
+      <x:c r="E45" s="52" t="str">
+        <x:v>Consultora Honda</x:v>
+      </x:c>
+      <x:c r="F45" s="52" t="str"/>
+      <x:c r="G45" s="52" t="str"/>
+      <x:c r="H45" s="52" t="str"/>
+      <x:c r="I45" s="52" t="str"/>
+      <x:c r="J45" s="52" t="str">
+        <x:v>https://www.instagram.com/mayaradahonda</x:v>
+      </x:c>
+      <x:c r="K45" s="52" t="str">
+        <x:v>Sem domínio de empregador confirmado</x:v>
+      </x:c>
+      <x:c r="L45" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M45" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. “Honda” é marca/produto e não identifica concessionária empregadora. Perfis ligados à Alagoas Motos estão associados ao respectivo domínio quando explícito; nos demais, sem domínio de empresa atribuído.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="56" customHeight="1">
+      <x:c r="A46" s="52" t="str">
+        <x:v>Débora Ávila</x:v>
+      </x:c>
+      <x:c r="B46" s="52" t="str">
+        <x:v>@debora_avila1980</x:v>
+      </x:c>
+      <x:c r="C46" s="52" t="str">
+        <x:v>CAOA Chery</x:v>
+      </x:c>
+      <x:c r="D46" s="52" t="str">
+        <x:v>caoa.com.br (grupo; unidade do lead não confirmada)</x:v>
+      </x:c>
+      <x:c r="E46" s="52" t="str">
+        <x:v>Executiva de Vendas</x:v>
+      </x:c>
+      <x:c r="F46" s="52" t="str"/>
+      <x:c r="G46" s="52" t="str"/>
+      <x:c r="H46" s="52" t="str"/>
+      <x:c r="I46" s="52" t="str">
+        <x:v>https://www.caoa.com.br/</x:v>
+      </x:c>
+      <x:c r="J46" s="52" t="str">
+        <x:v>https://www.instagram.com/debora_avila1980</x:v>
+      </x:c>
+      <x:c r="K46" s="52" t="str">
+        <x:v>Domínio identificado; vínculo/unidade individual parcial ou pendente</x:v>
+      </x:c>
+      <x:c r="L46" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M46" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Somente marca/grupo identificados; concessionária empregadora específica não confirmada.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="56" customHeight="1">
+      <x:c r="A47" s="52" t="str">
+        <x:v>Tiago Ripoli</x:v>
+      </x:c>
+      <x:c r="B47" s="52" t="str">
+        <x:v>@tiago_ripoli</x:v>
+      </x:c>
+      <x:c r="C47" s="52" t="str">
+        <x:v>Volkswagen</x:v>
+      </x:c>
+      <x:c r="D47" s="52" t="str">
+        <x:v>discasa.com.br</x:v>
+      </x:c>
+      <x:c r="E47" s="52" t="str">
+        <x:v>Profissional Volkswagen</x:v>
+      </x:c>
+      <x:c r="F47" s="52" t="str"/>
+      <x:c r="G47" s="52" t="str"/>
+      <x:c r="H47" s="52" t="str"/>
+      <x:c r="I47" s="52" t="str">
+        <x:v>https://www.discasa.com.br/fale-conosco/contato</x:v>
+      </x:c>
+      <x:c r="J47" s="52" t="str">
+        <x:v>https://www.instagram.com/tiago_ripoli</x:v>
+      </x:c>
+      <x:c r="K47" s="52" t="str">
+        <x:v>Domínio confirmado; vínculo da pessoa apoiado por fonte pública nominal</x:v>
+      </x:c>
+      <x:c r="L47" s="52" t="str">
+        <x:v>Publicação oficial da Discasa identifica Tiago Ripoli como consultor de vendas Volkswagen.</x:v>
+      </x:c>
+      <x:c r="M47" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Discasa confirma Tiago Ripoli como consultor em publicação oficial; telefone é canal geral de vendas.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="56" customHeight="1">
+      <x:c r="A48" s="52" t="str">
+        <x:v>Clayton consultor de veículos-BYD</x:v>
+      </x:c>
+      <x:c r="B48" s="52" t="str">
+        <x:v>@tomclay500</x:v>
+      </x:c>
+      <x:c r="C48" s="52" t="str">
+        <x:v>BYD</x:v>
+      </x:c>
+      <x:c r="D48" s="52" t="str">
+        <x:v>vitoriamotorsbyd.com.br (concessionária; pessoa/unidade a confirmar)</x:v>
+      </x:c>
+      <x:c r="E48" s="52" t="str">
+        <x:v>Consultor de Veículos</x:v>
+      </x:c>
+      <x:c r="F48" s="52" t="str"/>
+      <x:c r="G48" s="52" t="str"/>
+      <x:c r="H48" s="52" t="str"/>
+      <x:c r="I48" s="52" t="str">
+        <x:v>https://vitoriamotorsbyd.com.br/</x:v>
+      </x:c>
+      <x:c r="J48" s="52" t="str">
+        <x:v>https://www.instagram.com/tomclay500</x:v>
+      </x:c>
+      <x:c r="K48" s="52" t="str">
+        <x:v>Domínio identificado; vínculo/unidade individual parcial ou pendente</x:v>
+      </x:c>
+      <x:c r="L48" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M48" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Site oficial da Vitória Motors BYD. Perfil menciona consultoria BYD, mas nome completo/ligação à unidade não foram confirmados.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="56" customHeight="1">
+      <x:c r="A49" s="52" t="str">
+        <x:v>LEONARDO - ALAGOAS MOTOS</x:v>
+      </x:c>
+      <x:c r="B49" s="52" t="str">
+        <x:v>@leonardo082_honda</x:v>
+      </x:c>
+      <x:c r="C49" s="52" t="str">
+        <x:v>Alagoas Motos</x:v>
+      </x:c>
+      <x:c r="D49" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="E49" s="52" t="str">
+        <x:v>Especialista em Financiamento</x:v>
+      </x:c>
+      <x:c r="F49" s="52" t="str"/>
+      <x:c r="G49" s="52" t="str"/>
+      <x:c r="H49" s="52" t="str">
+        <x:v>(82) 3539-8605; WhatsApp geral (82) 99996-0571 — site oficial</x:v>
+      </x:c>
+      <x:c r="I49" s="52" t="str">
+        <x:v>https://alagoasmotos.com.br/</x:v>
+      </x:c>
+      <x:c r="J49" s="52" t="str">
+        <x:v>https://www.instagram.com/leonardo082_honda</x:v>
+      </x:c>
+      <x:c r="K49" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L49" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M49" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Site oficial Honda; lista Arapiraca, Maceió e União dos Palmares (3 lojas em AL). LinkedIn corporativo informa vínculo com Pernambuco Motos e outras unidades do grupo, mas validar se a prospecção será pela empresa local ou grupo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="56" customHeight="1">
+      <x:c r="A50" s="52" t="str">
+        <x:v>Wagner Fitzner</x:v>
+      </x:c>
+      <x:c r="B50" s="52" t="str">
+        <x:v>@entendendo.consorciohonda</x:v>
+      </x:c>
+      <x:c r="C50" s="52" t="str">
+        <x:v>Consórcio Honda</x:v>
+      </x:c>
+      <x:c r="D50" s="52" t="str"/>
+      <x:c r="E50" s="52" t="str">
+        <x:v>Profissional de Vendas e Gestão</x:v>
+      </x:c>
+      <x:c r="F50" s="52" t="str"/>
+      <x:c r="G50" s="52" t="str"/>
+      <x:c r="H50" s="52" t="str"/>
+      <x:c r="I50" s="52" t="str"/>
+      <x:c r="J50" s="52" t="str">
+        <x:v>https://www.instagram.com/entendendo.consorciohonda</x:v>
+      </x:c>
+      <x:c r="K50" s="52" t="str">
+        <x:v>Sem domínio de empregador confirmado</x:v>
+      </x:c>
+      <x:c r="L50" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M50" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. “Honda” é marca/produto e não identifica concessionária empregadora. Perfis ligados à Alagoas Motos estão associados ao respectivo domínio quando explícito; nos demais, sem domínio de empresa atribuído.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="56" customHeight="1">
+      <x:c r="A51" s="52" t="str">
+        <x:v>Rosi Firmino</x:v>
+      </x:c>
+      <x:c r="B51" s="52" t="str">
+        <x:v>@rosi.firmino1</x:v>
+      </x:c>
+      <x:c r="C51" s="52" t="str">
+        <x:v>Clovinho Veículos</x:v>
+      </x:c>
+      <x:c r="D51" s="52" t="str">
+        <x:v>clovinhoveiculos.com.br</x:v>
+      </x:c>
+      <x:c r="E51" s="52" t="str">
+        <x:v>Empresária automotiva</x:v>
+      </x:c>
+      <x:c r="F51" s="52" t="str"/>
+      <x:c r="G51" s="52" t="str"/>
+      <x:c r="H51" s="52" t="str">
+        <x:v>(27) 3113-5553; WhatsApp corporativo (27) 99923-5553 — site oficial</x:v>
+      </x:c>
+      <x:c r="I51" s="52" t="str">
+        <x:v>https://clovinhoveiculos.com.br/</x:v>
+      </x:c>
+      <x:c r="J51" s="52" t="str">
+        <x:v>https://www.instagram.com/rosi.firmino1</x:v>
+      </x:c>
+      <x:c r="K51" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L51" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M51" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Site oficial de revenda de seminovos em Colatina/ES com variedade de marcas; não é concessionária monomarca autorizada.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="56" customHeight="1">
+      <x:c r="A52" s="52" t="str">
+        <x:v>Nathalia Nispeche | Executiva de vendas | GAC JAVEP</x:v>
+      </x:c>
+      <x:c r="B52" s="52" t="str">
+        <x:v>@nathnispeche</x:v>
+      </x:c>
+      <x:c r="C52" s="52" t="str">
+        <x:v>GAC JAVEP</x:v>
+      </x:c>
+      <x:c r="D52" s="52" t="str">
+        <x:v>javepgac.com.br</x:v>
+      </x:c>
+      <x:c r="E52" s="52" t="str">
+        <x:v>Executiva de Vendas</x:v>
+      </x:c>
+      <x:c r="F52" s="52" t="str"/>
+      <x:c r="G52" s="52" t="str"/>
+      <x:c r="H52" s="52" t="str"/>
+      <x:c r="I52" s="52" t="str">
+        <x:v>https://javepgac.com.br/sobre-nos</x:v>
+      </x:c>
+      <x:c r="J52" s="52" t="str">
+        <x:v>https://www.instagram.com/nathnispeche</x:v>
+      </x:c>
+      <x:c r="K52" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L52" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M52" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Site Javep GAC confirma concessionária autorizada e unidades em SP. A página da empresa deve ser cruzada com a localização atual da lead; não prova vínculo individual.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="56" customHeight="1">
+      <x:c r="A53" s="52" t="str">
+        <x:v>Bruna Fernandes Cardoso</x:v>
+      </x:c>
+      <x:c r="B53" s="52" t="str">
+        <x:v>@brunafeh</x:v>
+      </x:c>
+      <x:c r="C53" s="52" t="str">
+        <x:v>Empresa não identificada na bio</x:v>
+      </x:c>
+      <x:c r="D53" s="52" t="str"/>
+      <x:c r="E53" s="52" t="str">
+        <x:v>Liderança em CRM e Marketing</x:v>
+      </x:c>
+      <x:c r="F53" s="52" t="str"/>
+      <x:c r="G53" s="52" t="str"/>
+      <x:c r="H53" s="52" t="str"/>
+      <x:c r="I53" s="52" t="str"/>
+      <x:c r="J53" s="52" t="str">
+        <x:v>https://www.instagram.com/brunafeh</x:v>
+      </x:c>
+      <x:c r="K53" s="52" t="str">
+        <x:v>Sem domínio de empregador confirmado</x:v>
+      </x:c>
+      <x:c r="L53" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M53" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Empresa não identificável pelo nome/URL disponíveis no registro. Precisa pedir empregador/unidade ao lead antes de procurar canais corporativos.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="56" customHeight="1">
+      <x:c r="A54" s="52" t="str">
+        <x:v>Representante comercial</x:v>
+      </x:c>
+      <x:c r="B54" s="52" t="str">
+        <x:v>@carolina_brazzo</x:v>
+      </x:c>
+      <x:c r="C54" s="52" t="str">
+        <x:v>Brazzo / Mobato</x:v>
+      </x:c>
+      <x:c r="D54" s="52" t="str">
+        <x:v>brazzo.com.br</x:v>
+      </x:c>
+      <x:c r="E54" s="52" t="str">
+        <x:v>Representante Comercial</x:v>
+      </x:c>
+      <x:c r="F54" s="52" t="str"/>
+      <x:c r="G54" s="52" t="str"/>
+      <x:c r="H54" s="52" t="str"/>
+      <x:c r="I54" s="52" t="str">
+        <x:v>https://brazzo.com.br/</x:v>
+      </x:c>
+      <x:c r="J54" s="52" t="str">
+        <x:v>https://www.instagram.com/carolina_brazzo</x:v>
+      </x:c>
+      <x:c r="K54" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L54" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M54" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Empresa fornecedora do setor (não concessionária prospect). Não há evidência pública suficiente de cargo/vínculo para este perfil.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="56" customHeight="1">
+      <x:c r="A55" s="52" t="str">
+        <x:v>Lucas Ricardo Belizário</x:v>
+      </x:c>
+      <x:c r="B55" s="52" t="str">
+        <x:v>@lucasricardobelizario</x:v>
+      </x:c>
+      <x:c r="C55" s="52" t="str">
+        <x:v>Brazzo</x:v>
+      </x:c>
+      <x:c r="D55" s="52" t="str">
+        <x:v>brazzo.com.br</x:v>
+      </x:c>
+      <x:c r="E55" s="52" t="str">
+        <x:v>Gestão de Vendas</x:v>
+      </x:c>
+      <x:c r="F55" s="52" t="str"/>
+      <x:c r="G55" s="52" t="str"/>
+      <x:c r="H55" s="52" t="str"/>
+      <x:c r="I55" s="52" t="str">
+        <x:v>https://www.linkedin.com/company/brazzo/</x:v>
+      </x:c>
+      <x:c r="J55" s="52" t="str">
+        <x:v>https://www.instagram.com/lucasricardobelizario</x:v>
+      </x:c>
+      <x:c r="K55" s="52" t="str">
+        <x:v>Domínio da empresa identificado; validar vínculo atual da pessoa</x:v>
+      </x:c>
+      <x:c r="L55" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M55" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Perfil corporativo público lista brazzo.com.br e a empresa como fornecedora do setor automotivo; não é conta cliente concessionária.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="56" customHeight="1">
+      <x:c r="A56" s="52" t="str">
+        <x:v>Thiago Ferreira</x:v>
+      </x:c>
+      <x:c r="B56" s="52" t="str">
+        <x:v>@thiago.bmw.motorrad</x:v>
+      </x:c>
+      <x:c r="C56" s="52" t="str">
+        <x:v>BMW Motorrad (empregador/unidade não explicitados na bio)</x:v>
+      </x:c>
+      <x:c r="D56" s="52" t="str"/>
+      <x:c r="E56" s="52" t="str">
+        <x:v>12 anos de Experiência em concessionárias 🎖️
+Executivo de vendas BMW Motorrad 🇩🇪
+Motocicletas BMW Zero km🛵
+Motocicletas Seminovas Multimarcas🏍️</x:v>
+      </x:c>
+      <x:c r="F56" s="52" t="str"/>
+      <x:c r="G56" s="52" t="str"/>
+      <x:c r="H56" s="52" t="str"/>
+      <x:c r="I56" s="52" t="str"/>
+      <x:c r="J56" s="52" t="str">
+        <x:v>https://www.instagram.com/thiago.bmw.motorrad</x:v>
+      </x:c>
+      <x:c r="K56" s="52" t="str">
+        <x:v>Sem domínio de empregador confirmado</x:v>
+      </x:c>
+      <x:c r="L56" s="52" t="str">
+        <x:v>Cargo/vínculo baseado na bio ou conteúdo público do próprio perfil; site corporativo confirma a empresa, não necessariamente a pessoa.</x:v>
+      </x:c>
+      <x:c r="M56" s="52" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. A bio indica BMW Motorrad, mas não informa concessionária/unidade. Não atribuí BM Rio: resultados para outros perfis Thiago Ferreira não correspondem ao mesmo @.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="56" customHeight="1">
+      <x:c r="A57" s="53" t="str">
+        <x:v>Luis Claudio Pinheiro</x:v>
+      </x:c>
+      <x:c r="B57" s="53" t="str">
+        <x:v>@luisclaudiopinheiro</x:v>
+      </x:c>
+      <x:c r="C57" s="53" t="str">
+        <x:v>BM Rio / BMW Motorrad (bio)</x:v>
+      </x:c>
+      <x:c r="D57" s="53" t="str">
+        <x:v>bmwrio.com.br; bmw-motorrad.com.br (página da concessionária)</x:v>
+      </x:c>
+      <x:c r="E57" s="53" t="str">
+        <x:v>Executivo de Vendas BMW Motorrad - BM RIO</x:v>
+      </x:c>
+      <x:c r="F57" s="53" t="str"/>
+      <x:c r="G57" s="53" t="str"/>
+      <x:c r="H57" s="53" t="str">
+        <x:v>+55 (21) 2042-4442; marketing@motorgroupvitoria.com.br — página oficial BMW Motorrad</x:v>
+      </x:c>
+      <x:c r="I57" s="53" t="str">
+        <x:v>https://www.bmw-motorrad.com.br/bmrio-botafogo-rj/pt/home.html</x:v>
+      </x:c>
+      <x:c r="J57" s="53" t="str">
+        <x:v>https://www.instagram.com/luisclaudiopinheiro</x:v>
+      </x:c>
+      <x:c r="K57" s="53" t="str">
+        <x:v>Domínio confirmado; vínculo da pessoa apoiado por fonte pública nominal</x:v>
+      </x:c>
+      <x:c r="L57" s="53" t="str">
+        <x:v>Bio do próprio perfil identifica BM RIO; página oficial BMW confirma concessionária e canais gerais.</x:v>
+      </x:c>
+      <x:c r="M57" s="53" t="str">
+        <x:v>Nenhum celular individual publicado confirmado nesta pesquisa. Bio indica BM RIO. Telefone +55 (21) 2042-4442 e marketing@motorgroupvitoria.com.br são canais gerais/corporativos, não pessoais.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:M1"/>
+    <x:mergeCell ref="A2:M2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc2f2910bece4ff5"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="52" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="46" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="66" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="30" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="52" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="92" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="209" t="str">
+        <x:v>Data Stone · busca de empresas por domínio</x:v>
+      </x:c>
+      <x:c r="B1" s="209"/>
+      <x:c r="C1" s="209"/>
+      <x:c r="D1" s="209"/>
+      <x:c r="E1" s="209"/>
+      <x:c r="F1" s="209"/>
+      <x:c r="G1" s="209"/>
+      <x:c r="H1" s="209"/>
+    </x:row>
+    <x:row r="2" ht="36" customHeight="1">
+      <x:c r="A2" s="6" t="str">
+        <x:v>25 domínios consultados via API /company/list/?domain=. A resposta pode ser ampla; apenas correspondências nominais plausíveis estão listadas como CNPJ candidato. Situação ativa e vínculo individual não foram confirmados nesta etapa. Documentação: https://docs.datastone.com.br/api</x:v>
+      </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+      <x:c r="H2" s="6"/>
+    </x:row>
+    <x:row r="5" ht="42" customHeight="1">
+      <x:c r="A5" s="226" t="str">
+        <x:v>Domínio consultado na Data Stone</x:v>
+      </x:c>
+      <x:c r="B5" s="226" t="str">
+        <x:v>Empresa(s) associadas aos leads</x:v>
+      </x:c>
+      <x:c r="C5" s="226" t="str">
+        <x:v>Resultados da API</x:v>
+      </x:c>
+      <x:c r="D5" s="226" t="str">
+        <x:v>CNPJ candidato(s) por nome</x:v>
+      </x:c>
+      <x:c r="E5" s="226" t="str">
+        <x:v>Razão social / nome fantasia correspondente</x:v>
+      </x:c>
+      <x:c r="F5" s="226" t="str">
+        <x:v>Cidade(s) / UF</x:v>
+      </x:c>
+      <x:c r="G5" s="226" t="str">
+        <x:v>Status da correspondência</x:v>
+      </x:c>
+      <x:c r="H5" s="226" t="str">
+        <x:v>Observação</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="52" customHeight="1">
+      <x:c r="A6" s="51" t="str">
+        <x:v>pinhoveiculos.com</x:v>
+      </x:c>
+      <x:c r="B6" s="51" t="str">
+        <x:v>Pinho Concessionária de Seminovos / Grupo S Pinho</x:v>
+      </x:c>
+      <x:c r="C6" s="51" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="D6" s="204" t="str">
+        <x:v>CNPJ: 10932867000139</x:v>
+      </x:c>
+      <x:c r="E6" s="51" t="str">
+        <x:v>PINHO COMERCIAL AL DE VEICULOS LTDA / PINHO CONCESSIONARIA DE SEMI NOVOS</x:v>
+      </x:c>
+      <x:c r="F6" s="51" t="str">
+        <x:v>RIO PARDO, RS</x:v>
+      </x:c>
+      <x:c r="G6" s="51" t="str">
+        <x:v>Candidato nominal; confirmar CNPJ ativo e associação com o lead</x:v>
+      </x:c>
+      <x:c r="H6" s="51" t="str">
+        <x:v>A busca por domínio retornou vários registros/filiais. Foram retidos apenas nomes que coincidem com a empresa mencionada; isso não confirma vínculo da pessoa nem situação cadastral ativa.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="52" customHeight="1">
+      <x:c r="A7" s="52" t="str">
+        <x:v>tagveiculosdf.com.br</x:v>
+      </x:c>
+      <x:c r="B7" s="52" t="str">
+        <x:v>TAG Veículos</x:v>
+      </x:c>
+      <x:c r="C7" s="52" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D7" s="205" t="str"/>
+      <x:c r="E7" s="52" t="str"/>
+      <x:c r="F7" s="52" t="str"/>
+      <x:c r="G7" s="52" t="str">
+        <x:v>Nenhum resultado para esse domínio</x:v>
+      </x:c>
+      <x:c r="H7" s="52" t="str">
+        <x:v>A API não retornou registro para o domínio informado; isso não prova que a empresa não exista.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="52" customHeight="1">
+      <x:c r="A8" s="52" t="str">
+        <x:v>akautocenter.com.br</x:v>
+      </x:c>
+      <x:c r="B8" s="52" t="str">
+        <x:v>AK Auto Center</x:v>
+      </x:c>
+      <x:c r="C8" s="52" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D8" s="205" t="str">
+        <x:v>CNPJ: 07799835000100</x:v>
+      </x:c>
+      <x:c r="E8" s="52" t="str">
+        <x:v>SOUZA COMERCIO E SERVICOS AUTOMOTIVOS LTDA / A.K. AUTOCENTER</x:v>
+      </x:c>
+      <x:c r="F8" s="52" t="str">
+        <x:v>SAO PAULO, SP</x:v>
+      </x:c>
+      <x:c r="G8" s="52" t="str">
+        <x:v>Candidato nominal; confirmar CNPJ ativo e associação com o lead</x:v>
+      </x:c>
+      <x:c r="H8" s="52" t="str">
+        <x:v>A busca por domínio retornou vários registros/filiais. Foram retidos apenas nomes que coincidem com a empresa mencionada; isso não confirma vínculo da pessoa nem situação cadastral ativa.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="52" customHeight="1">
+      <x:c r="A9" s="52" t="str">
+        <x:v>proveiculosmanaus.com.br</x:v>
+      </x:c>
+      <x:c r="B9" s="52" t="str">
+        <x:v>Pro Veículos Manaus / Alugue na Pro / Alveam</x:v>
+      </x:c>
+      <x:c r="C9" s="52" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D9" s="205" t="str"/>
+      <x:c r="E9" s="52" t="str"/>
+      <x:c r="F9" s="52" t="str"/>
+      <x:c r="G9" s="52" t="str">
+        <x:v>Nenhum resultado para esse domínio</x:v>
+      </x:c>
+      <x:c r="H9" s="52" t="str">
+        <x:v>A API não retornou registro para o domínio informado; isso não prova que a empresa não exista.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="52" customHeight="1">
+      <x:c r="A10" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="B10" s="52" t="str">
+        <x:v>Alagoas Motos; Concessionária não identificada na bio</x:v>
+      </x:c>
+      <x:c r="C10" s="52" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D10" s="205" t="str"/>
+      <x:c r="E10" s="52" t="str"/>
+      <x:c r="F10" s="52" t="str"/>
+      <x:c r="G10" s="52" t="str">
+        <x:v>Nenhum resultado para esse domínio</x:v>
+      </x:c>
+      <x:c r="H10" s="52" t="str">
+        <x:v>A API não retornou registro para o domínio informado; isso não prova que a empresa não exista.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="52" customHeight="1">
+      <x:c r="A11" s="52" t="str">
+        <x:v>kiasunmotors.com.br</x:v>
+      </x:c>
+      <x:c r="B11" s="52" t="str">
+        <x:v>Kia Sun Motors / Suzuki Sun Motors</x:v>
+      </x:c>
+      <x:c r="C11" s="52" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="D11" s="205" t="str">
+        <x:v>CNPJ: 73695397000580; 73695397000408; 73695397000157</x:v>
+      </x:c>
+      <x:c r="E11" s="52" t="str">
+        <x:v>SUN MOTORS COMERCIO DE VEICULOS LTDA</x:v>
+      </x:c>
+      <x:c r="F11" s="52" t="str">
+        <x:v>GRAMADO, RS; PORTO ALEGRE, RS</x:v>
+      </x:c>
+      <x:c r="G11" s="52" t="str">
+        <x:v>Candidato nominal; confirmar CNPJ ativo e associação com o lead</x:v>
+      </x:c>
+      <x:c r="H11" s="52" t="str">
+        <x:v>A busca por domínio retornou vários registros/filiais. Foram retidos apenas nomes que coincidem com a empresa mencionada; isso não confirma vínculo da pessoa nem situação cadastral ativa.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="52" customHeight="1">
+      <x:c r="A12" s="52" t="str">
+        <x:v>primaviafiat.com.br</x:v>
+      </x:c>
+      <x:c r="B12" s="52" t="str">
+        <x:v>Primavia Fiat</x:v>
+      </x:c>
+      <x:c r="C12" s="52" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D12" s="205" t="str"/>
+      <x:c r="E12" s="52" t="str"/>
+      <x:c r="F12" s="52" t="str"/>
+      <x:c r="G12" s="52" t="str">
+        <x:v>Nenhum resultado para esse domínio</x:v>
+      </x:c>
+      <x:c r="H12" s="52" t="str">
+        <x:v>A API não retornou registro para o domínio informado; isso não prova que a empresa não exista.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="52" customHeight="1">
+      <x:c r="A13" s="52" t="str">
+        <x:v>grupoprimavia.com.br</x:v>
+      </x:c>
+      <x:c r="B13" s="52" t="str">
+        <x:v>Primavia Fiat</x:v>
+      </x:c>
+      <x:c r="C13" s="52" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D13" s="205" t="str">
+        <x:v>CNPJ: 21043592000956; 71145668000175; 21043592000522</x:v>
+      </x:c>
+      <x:c r="E13" s="52" t="str">
+        <x:v>PRIMAVIA MOTORS LTDA; PRIMAVIA VEICULOS LTDA; PRIMAVIA MOTORS LTDA / VIA MOTORS</x:v>
+      </x:c>
+      <x:c r="F13" s="52" t="str">
+        <x:v>BRASILIA, DF; UNAI, MG; ARAGUAINA, TO</x:v>
+      </x:c>
+      <x:c r="G13" s="52" t="str">
+        <x:v>Candidato nominal; confirmar CNPJ ativo e associação com o lead</x:v>
+      </x:c>
+      <x:c r="H13" s="52" t="str">
+        <x:v>A busca por domínio retornou vários registros/filiais. Foram retidos apenas nomes que coincidem com a empresa mencionada; isso não confirma vínculo da pessoa nem situação cadastral ativa.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="52" customHeight="1">
+      <x:c r="A14" s="52" t="str">
+        <x:v>yamahaoriginal.com.br</x:v>
+      </x:c>
+      <x:c r="B14" s="52" t="str">
+        <x:v>Original Yamaha</x:v>
+      </x:c>
+      <x:c r="C14" s="52" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D14" s="205" t="str"/>
+      <x:c r="E14" s="52" t="str"/>
+      <x:c r="F14" s="52" t="str"/>
+      <x:c r="G14" s="52" t="str">
+        <x:v>Nenhum resultado para esse domínio</x:v>
+      </x:c>
+      <x:c r="H14" s="52" t="str">
+        <x:v>A API não retornou registro para o domínio informado; isso não prova que a empresa não exista.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="52" customHeight="1">
+      <x:c r="A15" s="52" t="str">
+        <x:v>originalautos.com.br</x:v>
+      </x:c>
+      <x:c r="B15" s="52" t="str">
+        <x:v>Original Yamaha; Original São Luís; CAOA Chery Original São Luís; Original Autos; Renault Original São Luís; Fiat Original São Luís</x:v>
+      </x:c>
+      <x:c r="C15" s="52" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D15" s="205" t="str"/>
+      <x:c r="E15" s="52" t="str"/>
+      <x:c r="F15" s="52" t="str"/>
+      <x:c r="G15" s="52" t="str">
+        <x:v>Resultados sem correspondência nominal segura</x:v>
+      </x:c>
+      <x:c r="H15" s="52" t="str">
+        <x:v>A consulta trouxe registros, mas nenhum nome fantasia/razão social bateu com segurança com a empresa do lead.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="52" customHeight="1">
+      <x:c r="A16" s="52" t="str">
+        <x:v>grupogama.com.br</x:v>
+      </x:c>
+      <x:c r="B16" s="52" t="str">
+        <x:v>Grupo Gama</x:v>
+      </x:c>
+      <x:c r="C16" s="52" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D16" s="205" t="str"/>
+      <x:c r="E16" s="52" t="str"/>
+      <x:c r="F16" s="52" t="str"/>
+      <x:c r="G16" s="52" t="str">
+        <x:v>Resultados sem correspondência nominal segura</x:v>
+      </x:c>
+      <x:c r="H16" s="52" t="str">
+        <x:v>A consulta trouxe registros, mas nenhum nome fantasia/razão social bateu com segurança com a empresa do lead.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="52" customHeight="1">
+      <x:c r="A17" s="52" t="str">
+        <x:v>quevendas.com.br</x:v>
+      </x:c>
+      <x:c r="B17" s="52" t="str">
+        <x:v>Q Vendas</x:v>
+      </x:c>
+      <x:c r="C17" s="52" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D17" s="205" t="str"/>
+      <x:c r="E17" s="52" t="str"/>
+      <x:c r="F17" s="52" t="str"/>
+      <x:c r="G17" s="52" t="str">
+        <x:v>Nenhum resultado para esse domínio</x:v>
+      </x:c>
+      <x:c r="H17" s="52" t="str">
+        <x:v>A API não retornou registro para o domínio informado; isso não prova que a empresa não exista.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="52" customHeight="1">
+      <x:c r="A18" s="52" t="str">
+        <x:v>drsulnissan.com.br</x:v>
+      </x:c>
+      <x:c r="B18" s="52" t="str">
+        <x:v>Nissan / Geely em Lages</x:v>
+      </x:c>
+      <x:c r="C18" s="52" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D18" s="205" t="str"/>
+      <x:c r="E18" s="52" t="str"/>
+      <x:c r="F18" s="52" t="str"/>
+      <x:c r="G18" s="52" t="str">
+        <x:v>Nenhum resultado para esse domínio</x:v>
+      </x:c>
+      <x:c r="H18" s="52" t="str">
+        <x:v>A API não retornou registro para o domínio informado; isso não prova que a empresa não exista.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="52" customHeight="1">
+      <x:c r="A19" s="52" t="str">
+        <x:v>italiana.com.br</x:v>
+      </x:c>
+      <x:c r="B19" s="52" t="str">
+        <x:v>Italiana Automóveis</x:v>
+      </x:c>
+      <x:c r="C19" s="52" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="D19" s="205" t="str">
+        <x:v>CNPJ: 02472105000179; 02472105000250; 02472105000330; 02472105000683; 02472105000764; 02472105000845; 02472105000926; 02472105001060</x:v>
+      </x:c>
+      <x:c r="E19" s="52" t="str">
+        <x:v>ITALIANA AUTOMOVEIS DO RECIFE LTDA.; ITALIANA AUTOMOVEIS DO RECIFE LTDA. / ITALIANA AUTOMOVEIS DO RECIFE LTDA</x:v>
+      </x:c>
+      <x:c r="F19" s="52" t="str">
+        <x:v>RECIFE, PE; CARUARU, PE</x:v>
+      </x:c>
+      <x:c r="G19" s="52" t="str">
+        <x:v>Candidato nominal; confirmar CNPJ ativo e associação com o lead</x:v>
+      </x:c>
+      <x:c r="H19" s="52" t="str">
+        <x:v>A busca por domínio retornou vários registros/filiais. Foram retidos apenas nomes que coincidem com a empresa mencionada; isso não confirma vínculo da pessoa nem situação cadastral ativa.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="52" customHeight="1">
+      <x:c r="A20" s="52" t="str">
+        <x:v>ahoffmannveiculos.com</x:v>
+      </x:c>
+      <x:c r="B20" s="52" t="str">
+        <x:v>Hoffmann Veículos</x:v>
+      </x:c>
+      <x:c r="C20" s="52" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D20" s="205" t="str"/>
+      <x:c r="E20" s="52" t="str"/>
+      <x:c r="F20" s="52" t="str"/>
+      <x:c r="G20" s="52" t="str">
+        <x:v>Nenhum resultado para esse domínio</x:v>
+      </x:c>
+      <x:c r="H20" s="52" t="str">
+        <x:v>A API não retornou registro para o domínio informado; isso não prova que a empresa não exista.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="52" customHeight="1">
+      <x:c r="A21" s="52" t="str">
+        <x:v>eurobarrafiat.com.br</x:v>
+      </x:c>
+      <x:c r="B21" s="52" t="str">
+        <x:v>Grupo Euroaméricas</x:v>
+      </x:c>
+      <x:c r="C21" s="52" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D21" s="205" t="str"/>
+      <x:c r="E21" s="52" t="str"/>
+      <x:c r="F21" s="52" t="str"/>
+      <x:c r="G21" s="52" t="str">
+        <x:v>Nenhum resultado para esse domínio</x:v>
+      </x:c>
+      <x:c r="H21" s="52" t="str">
+        <x:v>A API não retornou registro para o domínio informado; isso não prova que a empresa não exista.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="52" customHeight="1">
+      <x:c r="A22" s="52" t="str">
+        <x:v>consorcionacionalhonda.com.br</x:v>
+      </x:c>
+      <x:c r="B22" s="52" t="str">
+        <x:v>Consórcio Honda</x:v>
+      </x:c>
+      <x:c r="C22" s="52" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D22" s="205" t="str"/>
+      <x:c r="E22" s="52" t="str"/>
+      <x:c r="F22" s="52" t="str"/>
+      <x:c r="G22" s="52" t="str">
+        <x:v>Nenhum resultado para esse domínio</x:v>
+      </x:c>
+      <x:c r="H22" s="52" t="str">
+        <x:v>A API não retornou registro para o domínio informado; isso não prova que a empresa não exista.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="52" customHeight="1">
+      <x:c r="A23" s="52" t="str">
+        <x:v>caoa.com.br</x:v>
+      </x:c>
+      <x:c r="B23" s="52" t="str">
+        <x:v>CAOA Chery</x:v>
+      </x:c>
+      <x:c r="C23" s="52" t="n">
+        <x:v>804</x:v>
+      </x:c>
+      <x:c r="D23" s="205" t="str"/>
+      <x:c r="E23" s="52" t="str"/>
+      <x:c r="F23" s="52" t="str"/>
+      <x:c r="G23" s="52" t="str">
+        <x:v>Resposta ampla; sem CNPJ atribuído</x:v>
+      </x:c>
+      <x:c r="H23" s="52" t="str">
+        <x:v>A consulta trouxe muitos resultados não específicos. Não atribuí nenhum deles ao lead.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="52" customHeight="1">
+      <x:c r="A24" s="52" t="str">
+        <x:v>discasa.com.br</x:v>
+      </x:c>
+      <x:c r="B24" s="52" t="str">
+        <x:v>Volkswagen</x:v>
+      </x:c>
+      <x:c r="C24" s="52" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="D24" s="205" t="str">
+        <x:v>CNPJ: 59599134000113; 59599134000202; 59599134000385; 59599134000466</x:v>
+      </x:c>
+      <x:c r="E24" s="52" t="str">
+        <x:v>DISCASA-DISTRIBUIDORA SAOCARLENSE DE AUTOMOVEIS LTDA / DISCASA; DISCASA-DISTRIBUIDORA SAOCARLENSE DE AUTOMOVEIS LTDA</x:v>
+      </x:c>
+      <x:c r="F24" s="52" t="str">
+        <x:v>SAO CARLOS, SP; PORTO FERREIRA, SP</x:v>
+      </x:c>
+      <x:c r="G24" s="52" t="str">
+        <x:v>Candidato nominal; confirmar CNPJ ativo e associação com o lead</x:v>
+      </x:c>
+      <x:c r="H24" s="52" t="str">
+        <x:v>A busca por domínio retornou vários registros/filiais. Foram retidos apenas nomes que coincidem com a empresa mencionada; isso não confirma vínculo da pessoa nem situação cadastral ativa.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="52" customHeight="1">
+      <x:c r="A25" s="52" t="str">
+        <x:v>vitoriamotorsbyd.com.br</x:v>
+      </x:c>
+      <x:c r="B25" s="52" t="str">
+        <x:v>BYD</x:v>
+      </x:c>
+      <x:c r="C25" s="52" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D25" s="205" t="str"/>
+      <x:c r="E25" s="52" t="str"/>
+      <x:c r="F25" s="52" t="str"/>
+      <x:c r="G25" s="52" t="str">
+        <x:v>Nenhum resultado para esse domínio</x:v>
+      </x:c>
+      <x:c r="H25" s="52" t="str">
+        <x:v>A API não retornou registro para o domínio informado; isso não prova que a empresa não exista.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="52" customHeight="1">
+      <x:c r="A26" s="52" t="str">
+        <x:v>clovinhoveiculos.com.br</x:v>
+      </x:c>
+      <x:c r="B26" s="52" t="str">
+        <x:v>Clovinho Veículos</x:v>
+      </x:c>
+      <x:c r="C26" s="52" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D26" s="205" t="str"/>
+      <x:c r="E26" s="52" t="str"/>
+      <x:c r="F26" s="52" t="str"/>
+      <x:c r="G26" s="52" t="str">
+        <x:v>Nenhum resultado para esse domínio</x:v>
+      </x:c>
+      <x:c r="H26" s="52" t="str">
+        <x:v>A API não retornou registro para o domínio informado; isso não prova que a empresa não exista.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="52" customHeight="1">
+      <x:c r="A27" s="52" t="str">
+        <x:v>javepgac.com.br</x:v>
+      </x:c>
+      <x:c r="B27" s="52" t="str">
+        <x:v>GAC JAVEP</x:v>
+      </x:c>
+      <x:c r="C27" s="52" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D27" s="205" t="str"/>
+      <x:c r="E27" s="52" t="str"/>
+      <x:c r="F27" s="52" t="str"/>
+      <x:c r="G27" s="52" t="str">
+        <x:v>Nenhum resultado para esse domínio</x:v>
+      </x:c>
+      <x:c r="H27" s="52" t="str">
+        <x:v>A API não retornou registro para o domínio informado; isso não prova que a empresa não exista.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="52" customHeight="1">
+      <x:c r="A28" s="52" t="str">
+        <x:v>brazzo.com.br</x:v>
+      </x:c>
+      <x:c r="B28" s="52" t="str">
+        <x:v>Brazzo / Mobato; Brazzo</x:v>
+      </x:c>
+      <x:c r="C28" s="52" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="D28" s="205" t="str"/>
+      <x:c r="E28" s="52" t="str"/>
+      <x:c r="F28" s="52" t="str"/>
+      <x:c r="G28" s="52" t="str">
+        <x:v>Resultados sem correspondência nominal segura</x:v>
+      </x:c>
+      <x:c r="H28" s="52" t="str">
+        <x:v>A consulta trouxe registros, mas nenhum nome fantasia/razão social bateu com segurança com a empresa do lead.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="52" customHeight="1">
+      <x:c r="A29" s="52" t="str">
+        <x:v>bmwrio.com.br</x:v>
+      </x:c>
+      <x:c r="B29" s="52" t="str">
+        <x:v>BM Rio / BMW Motorrad (bio)</x:v>
+      </x:c>
+      <x:c r="C29" s="52" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D29" s="205" t="str"/>
+      <x:c r="E29" s="52" t="str"/>
+      <x:c r="F29" s="52" t="str"/>
+      <x:c r="G29" s="52" t="str">
+        <x:v>Nenhum resultado para esse domínio</x:v>
+      </x:c>
+      <x:c r="H29" s="52" t="str">
+        <x:v>A API não retornou registro para o domínio informado; isso não prova que a empresa não exista.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="52" customHeight="1">
+      <x:c r="A30" s="53" t="str">
+        <x:v>bmw-motorrad.com.br</x:v>
+      </x:c>
+      <x:c r="B30" s="53" t="str">
+        <x:v>BM Rio / BMW Motorrad (bio)</x:v>
+      </x:c>
+      <x:c r="C30" s="53" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D30" s="206" t="str"/>
+      <x:c r="E30" s="53" t="str"/>
+      <x:c r="F30" s="53" t="str"/>
+      <x:c r="G30" s="53" t="str">
+        <x:v>Nenhum resultado para esse domínio</x:v>
+      </x:c>
+      <x:c r="H30" s="53" t="str">
+        <x:v>A API não retornou registro para o domínio informado; isso não prova que a empresa não exista.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A2:H2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb957647b2fef4c03"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="54" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="90" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="35" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="35" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="80" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="209" t="str">
+        <x:v>Data Stone · resolução nominal de leads</x:v>
+      </x:c>
+      <x:c r="B1" s="209"/>
+      <x:c r="C1" s="209"/>
+      <x:c r="D1" s="209"/>
+      <x:c r="E1" s="209"/>
+      <x:c r="F1" s="209"/>
+      <x:c r="G1" s="209"/>
+    </x:row>
+    <x:row r="2" ht="36" customHeight="1">
+      <x:c r="A2" s="6" t="str">
+        <x:v>Busca B2B por empresa/CNPJ e cargo, seguida de tentativa de enriquecimento individual. Dados de contato só seriam preenchidos com correspondência nominal confirmada. Nesta rodada, a API não forneceu e-mail ou celular individual verificável. Documentação: https://docs.datastone.com.br/api/prospeccao-b2b/post_b2b_persons</x:v>
+      </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+    </x:row>
+    <x:row r="5" ht="42" customHeight="1">
+      <x:c r="A5" s="226" t="str">
+        <x:v>Lead</x:v>
+      </x:c>
+      <x:c r="B5" s="226" t="str">
+        <x:v>Instagram</x:v>
+      </x:c>
+      <x:c r="C5" s="226" t="str">
+        <x:v>Empresa/domain candidato</x:v>
+      </x:c>
+      <x:c r="D5" s="226" t="str">
+        <x:v>Resultado da busca nominal Data Stone</x:v>
+      </x:c>
+      <x:c r="E5" s="226" t="str">
+        <x:v>E-mail individual retornado pela API</x:v>
+      </x:c>
+      <x:c r="F5" s="226" t="str">
+        <x:v>Celular individual retornado pela API</x:v>
+      </x:c>
+      <x:c r="G5" s="226" t="str">
+        <x:v>Interpretação / próximo passo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="56" customHeight="1">
+      <x:c r="A6" s="51" t="str">
+        <x:v>Thiago Pinho</x:v>
+      </x:c>
+      <x:c r="B6" s="51" t="str">
+        <x:v>@thiagopinhotiti</x:v>
+      </x:c>
+      <x:c r="C6" s="51" t="str">
+        <x:v>pinhoveiculos.com (link da bio; associação nominal pendente)</x:v>
+      </x:c>
+      <x:c r="D6" s="51" t="str">
+        <x:v>Empresa enriquecida por CNPJ; Data Stone retornou correspondências nominais “Thiago dos Santos Pinho” / “Thiago Pinho” com papéis de sócio-administrador, sócio e diretor. A tentativa de obter contato individual não concluiu dentro do tempo limite.</x:v>
+      </x:c>
+      <x:c r="E6" s="51" t="str"/>
+      <x:c r="F6" s="51" t="str"/>
+      <x:c r="G6" s="51" t="str">
+        <x:v>Contato individual não obtido; validar se as variantes de nome são a mesma pessoa.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="56" customHeight="1">
+      <x:c r="A7" s="52" t="str">
+        <x:v>Eltton Andradee</x:v>
+      </x:c>
+      <x:c r="B7" s="52" t="str">
+        <x:v>@elttonandradee</x:v>
+      </x:c>
+      <x:c r="C7" s="52" t="str">
+        <x:v>tagveiculosdf.com.br</x:v>
+      </x:c>
+      <x:c r="D7" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E7" s="52" t="str"/>
+      <x:c r="F7" s="52" t="str"/>
+      <x:c r="G7" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="56" customHeight="1">
+      <x:c r="A8" s="52" t="str">
+        <x:v>SANDRA CARVALHO ⛤</x:v>
+      </x:c>
+      <x:c r="B8" s="52" t="str">
+        <x:v>@sandra.carvalho0702</x:v>
+      </x:c>
+      <x:c r="C8" s="52" t="str">
+        <x:v>akautocenter.com.br</x:v>
+      </x:c>
+      <x:c r="D8" s="52" t="str">
+        <x:v>Busca B2B por dois CNPJs candidatos da AK Auto Center e cargos de direção/proprietária: 0 pessoas retornadas.</x:v>
+      </x:c>
+      <x:c r="E8" s="52" t="str"/>
+      <x:c r="F8" s="52" t="str"/>
+      <x:c r="G8" s="52" t="str">
+        <x:v>Nenhum contato individual pela API nesta rodada.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="56" customHeight="1">
+      <x:c r="A9" s="52" t="str">
+        <x:v>Jaime Campelo Bessa</x:v>
+      </x:c>
+      <x:c r="B9" s="52" t="str">
+        <x:v>@jaimedapro</x:v>
+      </x:c>
+      <x:c r="C9" s="52" t="str">
+        <x:v>proveiculosmanaus.com.br</x:v>
+      </x:c>
+      <x:c r="D9" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E9" s="52" t="str"/>
+      <x:c r="F9" s="52" t="str"/>
+      <x:c r="G9" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="56" customHeight="1">
+      <x:c r="A10" s="52" t="str">
+        <x:v>Dallyane Barbosa Costa</x:v>
+      </x:c>
+      <x:c r="B10" s="52" t="str">
+        <x:v>@dallyanecostahonda</x:v>
+      </x:c>
+      <x:c r="C10" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="D10" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E10" s="52" t="str"/>
+      <x:c r="F10" s="52" t="str"/>
+      <x:c r="G10" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="56" customHeight="1">
+      <x:c r="A11" s="52" t="str">
+        <x:v>Deyvid Bezerra</x:v>
+      </x:c>
+      <x:c r="B11" s="52" t="str">
+        <x:v>@deyvid.honda</x:v>
+      </x:c>
+      <x:c r="C11" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="D11" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E11" s="52" t="str"/>
+      <x:c r="F11" s="52" t="str"/>
+      <x:c r="G11" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="56" customHeight="1">
+      <x:c r="A12" s="52" t="str">
+        <x:v>Emerson Angelino Cavalcante</x:v>
+      </x:c>
+      <x:c r="B12" s="52" t="str">
+        <x:v>@emerson.honda</x:v>
+      </x:c>
+      <x:c r="C12" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="D12" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E12" s="52" t="str"/>
+      <x:c r="F12" s="52" t="str"/>
+      <x:c r="G12" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="56" customHeight="1">
+      <x:c r="A13" s="52" t="str">
+        <x:v>Jefferson Furstenau</x:v>
+      </x:c>
+      <x:c r="B13" s="52" t="str">
+        <x:v>@jefferson.sunmotors</x:v>
+      </x:c>
+      <x:c r="C13" s="52" t="str">
+        <x:v>kiasunmotors.com.br</x:v>
+      </x:c>
+      <x:c r="D13" s="52" t="str">
+        <x:v>Busca B2B por Sun Motors + cargos de direção/gerência: API respondeu 429 (limite temporário).</x:v>
+      </x:c>
+      <x:c r="E13" s="52" t="str"/>
+      <x:c r="F13" s="52" t="str"/>
+      <x:c r="G13" s="52" t="str">
+        <x:v>Consulta de pessoa inconclusiva; sem enriquecimento individual.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="56" customHeight="1">
+      <x:c r="A14" s="52" t="str">
+        <x:v>Bruno Bettéro</x:v>
+      </x:c>
+      <x:c r="B14" s="52" t="str">
+        <x:v>@brunobettero</x:v>
+      </x:c>
+      <x:c r="C14" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="D14" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E14" s="52" t="str"/>
+      <x:c r="F14" s="52" t="str"/>
+      <x:c r="G14" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="56" customHeight="1">
+      <x:c r="A15" s="52" t="str">
+        <x:v>Gesivam Lopes</x:v>
+      </x:c>
+      <x:c r="B15" s="52" t="str">
+        <x:v>@gesivamlopes</x:v>
+      </x:c>
+      <x:c r="C15" s="52" t="str">
+        <x:v>primaviafiat.com.br; grupoprimavia.com.br (grupo)</x:v>
+      </x:c>
+      <x:c r="D15" s="52" t="str">
+        <x:v>Buscas B2B por Primavia Motors/Primavia Veículos + Gerente de Vendas: API respondeu 429 (limite temporário).</x:v>
+      </x:c>
+      <x:c r="E15" s="52" t="str"/>
+      <x:c r="F15" s="52" t="str"/>
+      <x:c r="G15" s="52" t="str">
+        <x:v>Consulta de pessoa inconclusiva; sem enriquecimento individual.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="56" customHeight="1">
+      <x:c r="A16" s="52" t="str">
+        <x:v>Keyanny</x:v>
+      </x:c>
+      <x:c r="B16" s="52" t="str">
+        <x:v>@keyannyalves</x:v>
+      </x:c>
+      <x:c r="C16" s="52" t="str">
+        <x:v>yamahaoriginal.com.br; originalautos.com.br (grupo)</x:v>
+      </x:c>
+      <x:c r="D16" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E16" s="52" t="str"/>
+      <x:c r="F16" s="52" t="str"/>
+      <x:c r="G16" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="56" customHeight="1">
+      <x:c r="A17" s="52" t="str">
+        <x:v>Reinaldo R. Cardoso | Conteúdo Automotivo</x:v>
+      </x:c>
+      <x:c r="B17" s="52" t="str">
+        <x:v>@reicardoso</x:v>
+      </x:c>
+      <x:c r="C17" s="52" t="str"/>
+      <x:c r="D17" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E17" s="52" t="str"/>
+      <x:c r="F17" s="52" t="str"/>
+      <x:c r="G17" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="56" customHeight="1">
+      <x:c r="A18" s="52" t="str">
+        <x:v>Junior Mendes</x:v>
+      </x:c>
+      <x:c r="B18" s="52" t="str">
+        <x:v>@juniormendes___</x:v>
+      </x:c>
+      <x:c r="C18" s="52" t="str">
+        <x:v>originalautos.com.br</x:v>
+      </x:c>
+      <x:c r="D18" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E18" s="52" t="str"/>
+      <x:c r="F18" s="52" t="str"/>
+      <x:c r="G18" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="56" customHeight="1">
+      <x:c r="A19" s="52" t="str">
+        <x:v>Ana Angélica</x:v>
+      </x:c>
+      <x:c r="B19" s="52" t="str">
+        <x:v>@angelicaomena</x:v>
+      </x:c>
+      <x:c r="C19" s="52" t="str">
+        <x:v>grupogama.com.br</x:v>
+      </x:c>
+      <x:c r="D19" s="52" t="str">
+        <x:v>Busca B2B Data Stone por Grupo Gama + Gerente Comercial: 0 pessoas retornadas.</x:v>
+      </x:c>
+      <x:c r="E19" s="52" t="str"/>
+      <x:c r="F19" s="52" t="str"/>
+      <x:c r="G19" s="52" t="str">
+        <x:v>Não encontrado nesta consulta; não significa que a pessoa não exista na base.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="56" customHeight="1">
+      <x:c r="A20" s="52" t="str">
+        <x:v>Gessiane Nina| Original Caoa Chery</x:v>
+      </x:c>
+      <x:c r="B20" s="52" t="str">
+        <x:v>@gessiane.nina</x:v>
+      </x:c>
+      <x:c r="C20" s="52" t="str">
+        <x:v>originalautos.com.br</x:v>
+      </x:c>
+      <x:c r="D20" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E20" s="52" t="str"/>
+      <x:c r="F20" s="52" t="str"/>
+      <x:c r="G20" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="56" customHeight="1">
+      <x:c r="A21" s="52" t="str">
+        <x:v>Leandro Guimarães</x:v>
+      </x:c>
+      <x:c r="B21" s="52" t="str">
+        <x:v>@leandroguimaraesal</x:v>
+      </x:c>
+      <x:c r="C21" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="D21" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E21" s="52" t="str"/>
+      <x:c r="F21" s="52" t="str"/>
+      <x:c r="G21" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="56" customHeight="1">
+      <x:c r="A22" s="52" t="str">
+        <x:v>Wallas Oliveira</x:v>
+      </x:c>
+      <x:c r="B22" s="52" t="str">
+        <x:v>@wallasoliveira</x:v>
+      </x:c>
+      <x:c r="C22" s="52" t="str"/>
+      <x:c r="D22" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E22" s="52" t="str"/>
+      <x:c r="F22" s="52" t="str"/>
+      <x:c r="G22" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="56" customHeight="1">
+      <x:c r="A23" s="52" t="str">
+        <x:v>Lucas Abreu /Carros Seminovos</x:v>
+      </x:c>
+      <x:c r="B23" s="52" t="str">
+        <x:v>@lucas.babreu</x:v>
+      </x:c>
+      <x:c r="C23" s="52" t="str">
+        <x:v>originalautos.com.br</x:v>
+      </x:c>
+      <x:c r="D23" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E23" s="52" t="str"/>
+      <x:c r="F23" s="52" t="str"/>
+      <x:c r="G23" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="56" customHeight="1">
+      <x:c r="A24" s="52" t="str">
+        <x:v>Soljane Mendes</x:v>
+      </x:c>
+      <x:c r="B24" s="52" t="str">
+        <x:v>@antoniasolijane</x:v>
+      </x:c>
+      <x:c r="C24" s="52" t="str">
+        <x:v>originalautos.com.br</x:v>
+      </x:c>
+      <x:c r="D24" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E24" s="52" t="str"/>
+      <x:c r="F24" s="52" t="str"/>
+      <x:c r="G24" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="56" customHeight="1">
+      <x:c r="A25" s="52" t="str">
+        <x:v>Mineiro da Honda | Consórcio em Arapiraca</x:v>
+      </x:c>
+      <x:c r="B25" s="52" t="str">
+        <x:v>@izael_doconsorcio</x:v>
+      </x:c>
+      <x:c r="C25" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="D25" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E25" s="52" t="str"/>
+      <x:c r="F25" s="52" t="str"/>
+      <x:c r="G25" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="56" customHeight="1">
+      <x:c r="A26" s="52" t="str">
+        <x:v>FAGNÉ </x:v>
+      </x:c>
+      <x:c r="B26" s="52" t="str">
+        <x:v>@fagnerdahonda</x:v>
+      </x:c>
+      <x:c r="C26" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="D26" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E26" s="52" t="str"/>
+      <x:c r="F26" s="52" t="str"/>
+      <x:c r="G26" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="56" customHeight="1">
+      <x:c r="A27" s="52" t="str">
+        <x:v>Klebson Wesley | Consórcio Honda</x:v>
+      </x:c>
+      <x:c r="B27" s="52" t="str">
+        <x:v>@klebson_honda</x:v>
+      </x:c>
+      <x:c r="C27" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="D27" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E27" s="52" t="str"/>
+      <x:c r="F27" s="52" t="str"/>
+      <x:c r="G27" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="56" customHeight="1">
+      <x:c r="A28" s="52" t="str">
+        <x:v>CRYS DA HONDA / CONSÓRCIO HONDA 🏆🥇🙏</x:v>
+      </x:c>
+      <x:c r="B28" s="52" t="str">
+        <x:v>@crys_da_honda</x:v>
+      </x:c>
+      <x:c r="C28" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="D28" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E28" s="52" t="str"/>
+      <x:c r="F28" s="52" t="str"/>
+      <x:c r="G28" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="56" customHeight="1">
+      <x:c r="A29" s="52" t="str">
+        <x:v>GSerejo 🏅</x:v>
+      </x:c>
+      <x:c r="B29" s="52" t="str">
+        <x:v>@lennyserejo</x:v>
+      </x:c>
+      <x:c r="C29" s="52" t="str">
+        <x:v>originalautos.com.br</x:v>
+      </x:c>
+      <x:c r="D29" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E29" s="52" t="str"/>
+      <x:c r="F29" s="52" t="str"/>
+      <x:c r="G29" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="56" customHeight="1">
+      <x:c r="A30" s="52" t="str">
+        <x:v>Gelison Ramos | Consórcio Honda Brasil 🇧🇷</x:v>
+      </x:c>
+      <x:c r="B30" s="52" t="str">
+        <x:v>@gelisonhonda</x:v>
+      </x:c>
+      <x:c r="C30" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="D30" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E30" s="52" t="str"/>
+      <x:c r="F30" s="52" t="str"/>
+      <x:c r="G30" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="56" customHeight="1">
+      <x:c r="A31" s="52" t="str">
+        <x:v>Adrielle Bezerra</x:v>
+      </x:c>
+      <x:c r="B31" s="52" t="str">
+        <x:v>@adriellehondaa</x:v>
+      </x:c>
+      <x:c r="C31" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="D31" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E31" s="52" t="str"/>
+      <x:c r="F31" s="52" t="str"/>
+      <x:c r="G31" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="56" customHeight="1">
+      <x:c r="A32" s="52" t="str">
+        <x:v>Jô Vieira - 🚘Q Vendas🚘</x:v>
+      </x:c>
+      <x:c r="B32" s="52" t="str">
+        <x:v>@jovieira_qvendas</x:v>
+      </x:c>
+      <x:c r="C32" s="52" t="str">
+        <x:v>quevendas.com.br</x:v>
+      </x:c>
+      <x:c r="D32" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E32" s="52" t="str"/>
+      <x:c r="F32" s="52" t="str"/>
+      <x:c r="G32" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="56" customHeight="1">
+      <x:c r="A33" s="52" t="str">
+        <x:v>Elaine Brumati</x:v>
+      </x:c>
+      <x:c r="B33" s="52" t="str">
+        <x:v>@elainebrumati</x:v>
+      </x:c>
+      <x:c r="C33" s="52" t="str"/>
+      <x:c r="D33" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E33" s="52" t="str"/>
+      <x:c r="F33" s="52" t="str"/>
+      <x:c r="G33" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="56" customHeight="1">
+      <x:c r="A34" s="52" t="str">
+        <x:v>Weryka Samara/Consórcio Honda</x:v>
+      </x:c>
+      <x:c r="B34" s="52" t="str">
+        <x:v>@werykasamara_honda</x:v>
+      </x:c>
+      <x:c r="C34" s="52" t="str"/>
+      <x:c r="D34" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E34" s="52" t="str"/>
+      <x:c r="F34" s="52" t="str"/>
+      <x:c r="G34" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="56" customHeight="1">
+      <x:c r="A35" s="52" t="str">
+        <x:v>Paulo Borba</x:v>
+      </x:c>
+      <x:c r="B35" s="52" t="str">
+        <x:v>@borba.nissan</x:v>
+      </x:c>
+      <x:c r="C35" s="52" t="str">
+        <x:v>drsulnissan.com.br (unidade Nissan Lages; vínculo apoiado pela bio)</x:v>
+      </x:c>
+      <x:c r="D35" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E35" s="52" t="str"/>
+      <x:c r="F35" s="52" t="str"/>
+      <x:c r="G35" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="56" customHeight="1">
+      <x:c r="A36" s="52" t="str">
+        <x:v>Wendell Brandão | Consultor Honda 🏍️</x:v>
+      </x:c>
+      <x:c r="B36" s="52" t="str">
+        <x:v>@wendellhondaa</x:v>
+      </x:c>
+      <x:c r="C36" s="52" t="str"/>
+      <x:c r="D36" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E36" s="52" t="str"/>
+      <x:c r="F36" s="52" t="str"/>
+      <x:c r="G36" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="56" customHeight="1">
+      <x:c r="A37" s="52" t="str">
+        <x:v>Bruno Fernando</x:v>
+      </x:c>
+      <x:c r="B37" s="52" t="str">
+        <x:v>@bruno.fernando.fiatslz</x:v>
+      </x:c>
+      <x:c r="C37" s="52" t="str">
+        <x:v>originalautos.com.br</x:v>
+      </x:c>
+      <x:c r="D37" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E37" s="52" t="str"/>
+      <x:c r="F37" s="52" t="str"/>
+      <x:c r="G37" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="56" customHeight="1">
+      <x:c r="A38" s="52" t="str">
+        <x:v>Eduardo Pitta Pontual</x:v>
+      </x:c>
+      <x:c r="B38" s="52" t="str">
+        <x:v>@eduardopittapontual</x:v>
+      </x:c>
+      <x:c r="C38" s="52" t="str">
+        <x:v>italiana.com.br</x:v>
+      </x:c>
+      <x:c r="D38" s="52" t="str">
+        <x:v>Busca B2B por Italiana Automóveis + cargos de vendas: API respondeu 429 (limite temporário).</x:v>
+      </x:c>
+      <x:c r="E38" s="52" t="str"/>
+      <x:c r="F38" s="52" t="str"/>
+      <x:c r="G38" s="52" t="str">
+        <x:v>Consulta de pessoa inconclusiva; sem enriquecimento individual.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="56" customHeight="1">
+      <x:c r="A39" s="52" t="str">
+        <x:v>Alexandre Hoffmann</x:v>
+      </x:c>
+      <x:c r="B39" s="52" t="str">
+        <x:v>@ahoffmannveiculos</x:v>
+      </x:c>
+      <x:c r="C39" s="52" t="str">
+        <x:v>ahoffmannveiculos.com</x:v>
+      </x:c>
+      <x:c r="D39" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E39" s="52" t="str"/>
+      <x:c r="F39" s="52" t="str"/>
+      <x:c r="G39" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="56" customHeight="1">
+      <x:c r="A40" s="52" t="str">
+        <x:v>Luiz Henrique Tubarão</x:v>
+      </x:c>
+      <x:c r="B40" s="52" t="str">
+        <x:v>@luizhenriquetubarao</x:v>
+      </x:c>
+      <x:c r="C40" s="52" t="str">
+        <x:v>eurobarrafiat.com.br (loja Fiat do grupo)</x:v>
+      </x:c>
+      <x:c r="D40" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E40" s="52" t="str"/>
+      <x:c r="F40" s="52" t="str"/>
+      <x:c r="G40" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="56" customHeight="1">
+      <x:c r="A41" s="52" t="str">
+        <x:v>ALEXANDRE | CONSÓRCIO HONDA</x:v>
+      </x:c>
+      <x:c r="B41" s="52" t="str">
+        <x:v>@alexandrechonda</x:v>
+      </x:c>
+      <x:c r="C41" s="52" t="str"/>
+      <x:c r="D41" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E41" s="52" t="str"/>
+      <x:c r="F41" s="52" t="str"/>
+      <x:c r="G41" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="56" customHeight="1">
+      <x:c r="A42" s="52" t="str">
+        <x:v>Italo Antonio | Consórcio Honda | Moto 0KM 🏍️</x:v>
+      </x:c>
+      <x:c r="B42" s="52" t="str">
+        <x:v>@italodahonda082</x:v>
+      </x:c>
+      <x:c r="C42" s="52" t="str"/>
+      <x:c r="D42" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E42" s="52" t="str"/>
+      <x:c r="F42" s="52" t="str"/>
+      <x:c r="G42" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="56" customHeight="1">
+      <x:c r="A43" s="52" t="str">
+        <x:v>Guilherme Caetano</x:v>
+      </x:c>
+      <x:c r="B43" s="52" t="str">
+        <x:v>@guilherme.honda1</x:v>
+      </x:c>
+      <x:c r="C43" s="52" t="str"/>
+      <x:c r="D43" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E43" s="52" t="str"/>
+      <x:c r="F43" s="52" t="str"/>
+      <x:c r="G43" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="56" customHeight="1">
+      <x:c r="A44" s="52" t="str">
+        <x:v>Karoll cavalcante | Honda</x:v>
+      </x:c>
+      <x:c r="B44" s="52" t="str">
+        <x:v>@karollhonda</x:v>
+      </x:c>
+      <x:c r="C44" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="D44" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E44" s="52" t="str"/>
+      <x:c r="F44" s="52" t="str"/>
+      <x:c r="G44" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="56" customHeight="1">
+      <x:c r="A45" s="52" t="str">
+        <x:v>Mayara da Honda</x:v>
+      </x:c>
+      <x:c r="B45" s="52" t="str">
+        <x:v>@mayaradahonda</x:v>
+      </x:c>
+      <x:c r="C45" s="52" t="str"/>
+      <x:c r="D45" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E45" s="52" t="str"/>
+      <x:c r="F45" s="52" t="str"/>
+      <x:c r="G45" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="56" customHeight="1">
+      <x:c r="A46" s="52" t="str">
+        <x:v>Débora Ávila</x:v>
+      </x:c>
+      <x:c r="B46" s="52" t="str">
+        <x:v>@debora_avila1980</x:v>
+      </x:c>
+      <x:c r="C46" s="52" t="str">
+        <x:v>caoa.com.br (grupo; unidade do lead não confirmada)</x:v>
+      </x:c>
+      <x:c r="D46" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E46" s="52" t="str"/>
+      <x:c r="F46" s="52" t="str"/>
+      <x:c r="G46" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="56" customHeight="1">
+      <x:c r="A47" s="52" t="str">
+        <x:v>Tiago Ripoli</x:v>
+      </x:c>
+      <x:c r="B47" s="52" t="str">
+        <x:v>@tiago_ripoli</x:v>
+      </x:c>
+      <x:c r="C47" s="52" t="str">
+        <x:v>discasa.com.br</x:v>
+      </x:c>
+      <x:c r="D47" s="52" t="str">
+        <x:v>Busca B2B por Discasa + Consultor de Vendas: API respondeu 429 (limite temporário).</x:v>
+      </x:c>
+      <x:c r="E47" s="52" t="str"/>
+      <x:c r="F47" s="52" t="str"/>
+      <x:c r="G47" s="52" t="str">
+        <x:v>Consulta de pessoa inconclusiva; sem enriquecimento individual.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="56" customHeight="1">
+      <x:c r="A48" s="52" t="str">
+        <x:v>Clayton consultor de veículos-BYD</x:v>
+      </x:c>
+      <x:c r="B48" s="52" t="str">
+        <x:v>@tomclay500</x:v>
+      </x:c>
+      <x:c r="C48" s="52" t="str">
+        <x:v>vitoriamotorsbyd.com.br (concessionária; pessoa/unidade a confirmar)</x:v>
+      </x:c>
+      <x:c r="D48" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E48" s="52" t="str"/>
+      <x:c r="F48" s="52" t="str"/>
+      <x:c r="G48" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="56" customHeight="1">
+      <x:c r="A49" s="52" t="str">
+        <x:v>LEONARDO - ALAGOAS MOTOS</x:v>
+      </x:c>
+      <x:c r="B49" s="52" t="str">
+        <x:v>@leonardo082_honda</x:v>
+      </x:c>
+      <x:c r="C49" s="52" t="str">
+        <x:v>alagoasmotos.com.br</x:v>
+      </x:c>
+      <x:c r="D49" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E49" s="52" t="str"/>
+      <x:c r="F49" s="52" t="str"/>
+      <x:c r="G49" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="56" customHeight="1">
+      <x:c r="A50" s="52" t="str">
+        <x:v>Wagner Fitzner</x:v>
+      </x:c>
+      <x:c r="B50" s="52" t="str">
+        <x:v>@entendendo.consorciohonda</x:v>
+      </x:c>
+      <x:c r="C50" s="52" t="str"/>
+      <x:c r="D50" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E50" s="52" t="str"/>
+      <x:c r="F50" s="52" t="str"/>
+      <x:c r="G50" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="56" customHeight="1">
+      <x:c r="A51" s="52" t="str">
+        <x:v>Rosi Firmino</x:v>
+      </x:c>
+      <x:c r="B51" s="52" t="str">
+        <x:v>@rosi.firmino1</x:v>
+      </x:c>
+      <x:c r="C51" s="52" t="str">
+        <x:v>clovinhoveiculos.com.br</x:v>
+      </x:c>
+      <x:c r="D51" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E51" s="52" t="str"/>
+      <x:c r="F51" s="52" t="str"/>
+      <x:c r="G51" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="56" customHeight="1">
+      <x:c r="A52" s="52" t="str">
+        <x:v>Nathalia Nispeche | Executiva de vendas | GAC JAVEP</x:v>
+      </x:c>
+      <x:c r="B52" s="52" t="str">
+        <x:v>@nathnispeche</x:v>
+      </x:c>
+      <x:c r="C52" s="52" t="str">
+        <x:v>javepgac.com.br</x:v>
+      </x:c>
+      <x:c r="D52" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E52" s="52" t="str"/>
+      <x:c r="F52" s="52" t="str"/>
+      <x:c r="G52" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="56" customHeight="1">
+      <x:c r="A53" s="52" t="str">
+        <x:v>Bruna Fernandes Cardoso</x:v>
+      </x:c>
+      <x:c r="B53" s="52" t="str">
+        <x:v>@brunafeh</x:v>
+      </x:c>
+      <x:c r="C53" s="52" t="str"/>
+      <x:c r="D53" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E53" s="52" t="str"/>
+      <x:c r="F53" s="52" t="str"/>
+      <x:c r="G53" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="56" customHeight="1">
+      <x:c r="A54" s="52" t="str">
+        <x:v>Representante comercial</x:v>
+      </x:c>
+      <x:c r="B54" s="52" t="str">
+        <x:v>@carolina_brazzo</x:v>
+      </x:c>
+      <x:c r="C54" s="52" t="str">
+        <x:v>brazzo.com.br</x:v>
+      </x:c>
+      <x:c r="D54" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E54" s="52" t="str"/>
+      <x:c r="F54" s="52" t="str"/>
+      <x:c r="G54" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="56" customHeight="1">
+      <x:c r="A55" s="52" t="str">
+        <x:v>Lucas Ricardo Belizário</x:v>
+      </x:c>
+      <x:c r="B55" s="52" t="str">
+        <x:v>@lucasricardobelizario</x:v>
+      </x:c>
+      <x:c r="C55" s="52" t="str">
+        <x:v>brazzo.com.br</x:v>
+      </x:c>
+      <x:c r="D55" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E55" s="52" t="str"/>
+      <x:c r="F55" s="52" t="str"/>
+      <x:c r="G55" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="56" customHeight="1">
+      <x:c r="A56" s="52" t="str">
+        <x:v>Thiago Ferreira</x:v>
+      </x:c>
+      <x:c r="B56" s="52" t="str">
+        <x:v>@thiago.bmw.motorrad</x:v>
+      </x:c>
+      <x:c r="C56" s="52" t="str"/>
+      <x:c r="D56" s="52" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E56" s="52" t="str"/>
+      <x:c r="F56" s="52" t="str"/>
+      <x:c r="G56" s="52" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="56" customHeight="1">
+      <x:c r="A57" s="53" t="str">
+        <x:v>Luis Claudio Pinheiro</x:v>
+      </x:c>
+      <x:c r="B57" s="53" t="str">
+        <x:v>@luisclaudiopinheiro</x:v>
+      </x:c>
+      <x:c r="C57" s="53" t="str">
+        <x:v>bmwrio.com.br; bmw-motorrad.com.br (página da concessionária)</x:v>
+      </x:c>
+      <x:c r="D57" s="53" t="str">
+        <x:v>Não pesquisado individualmente na Data Stone nesta rodada.</x:v>
+      </x:c>
+      <x:c r="E57" s="53" t="str"/>
+      <x:c r="F57" s="53" t="str"/>
+      <x:c r="G57" s="53" t="str">
+        <x:v>Nenhum contato Data Stone confirmado. Use apenas o WhatsApp profissional público listado na aba Enriquecimento público, quando houver.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A2:G2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8858301452894c51"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>